<commit_message>
Sync from OneDrive: DSafarik_2026TimeTracking.xlsx [2026-04-09 15:25 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ctbuh.sharepoint.com/sites/Staff/Shared Documents/Research/Time Tracking/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2472" documentId="8_{0FDB2C51-E576-4C63-8BE8-7A83A2F616A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17A9DCC1-082C-476B-B842-88E1E5779000}"/>
+  <xr:revisionPtr revIDLastSave="2491" documentId="8_{0FDB2C51-E576-4C63-8BE8-7A83A2F616A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BAB8FD7-37D2-4404-A060-4C7BFB7F9FE7}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{0C10F557-92E5-4EB6-9E48-62A8B86D346C}"/>
+    <workbookView xWindow="28635" yWindow="-165" windowWidth="29130" windowHeight="17610" xr2:uid="{0C10F557-92E5-4EB6-9E48-62A8B86D346C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tracking" sheetId="1" r:id="rId1"/>
@@ -1433,11 +1433,11 @@
       </c>
       <c r="BS1" s="10">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="BT1" s="10">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BU1" s="10">
         <f t="shared" ref="BU1:CD2" si="7">SUM(BU$7:BU$1048576)</f>
@@ -2483,11 +2483,11 @@
       </c>
       <c r="BS2" s="10">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="BT2" s="10">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BU2" s="10">
         <f t="shared" si="7"/>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="BS3" s="10">
         <f t="shared" si="27"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="BT3" s="10">
         <f t="shared" si="27"/>
@@ -7199,7 +7199,7 @@
       </c>
       <c r="B7" s="11">
         <f>SUM(B8:B23)</f>
-        <v>162.75</v>
+        <v>167.25</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -8279,7 +8279,7 @@
       </c>
       <c r="B11" s="7">
         <f t="shared" si="41"/>
-        <v>31.5</v>
+        <v>32.5</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -8397,7 +8397,9 @@
       <c r="BR11" s="18">
         <v>1</v>
       </c>
-      <c r="BS11" s="18"/>
+      <c r="BS11" s="18">
+        <v>1</v>
+      </c>
       <c r="BT11" s="18"/>
       <c r="BU11" s="18"/>
       <c r="BV11" s="18"/>
@@ -10255,7 +10257,7 @@
       </c>
       <c r="B18" s="7">
         <f t="shared" si="41"/>
-        <v>0.3</v>
+        <v>1.3</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
@@ -10327,7 +10329,9 @@
       <c r="BP18" s="18"/>
       <c r="BQ18" s="18"/>
       <c r="BR18" s="18"/>
-      <c r="BS18" s="18"/>
+      <c r="BS18" s="18">
+        <v>1</v>
+      </c>
       <c r="BT18" s="18"/>
       <c r="BU18" s="18"/>
       <c r="BV18" s="18"/>
@@ -11080,7 +11084,7 @@
       </c>
       <c r="B21" s="7">
         <f t="shared" si="41"/>
-        <v>18.25</v>
+        <v>20.75</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
@@ -11188,8 +11192,12 @@
       <c r="BR21" s="18">
         <v>0.25</v>
       </c>
-      <c r="BS21" s="18"/>
-      <c r="BT21" s="18"/>
+      <c r="BS21" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="BT21" s="18">
+        <v>2</v>
+      </c>
       <c r="BU21" s="18"/>
       <c r="BV21" s="18"/>
       <c r="BW21" s="18"/>
@@ -13851,7 +13859,7 @@
       </c>
       <c r="B31" s="7">
         <f t="shared" ref="B31:B40" si="42">SUM($C31:$XFD31)</f>
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
@@ -13996,8 +14004,12 @@
         <v>2</v>
       </c>
       <c r="BR31" s="18"/>
-      <c r="BS31" s="18"/>
-      <c r="BT31" s="18"/>
+      <c r="BS31" s="18">
+        <v>1</v>
+      </c>
+      <c r="BT31" s="18">
+        <v>2</v>
+      </c>
       <c r="BU31" s="18"/>
       <c r="BV31" s="18"/>
       <c r="BW31" s="18"/>
@@ -14466,7 +14478,7 @@
       </c>
       <c r="B33" s="7">
         <f t="shared" si="42"/>
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
@@ -14580,8 +14592,12 @@
       <c r="BR33" s="18">
         <v>2</v>
       </c>
-      <c r="BS33" s="18"/>
-      <c r="BT33" s="18"/>
+      <c r="BS33" s="18">
+        <v>1</v>
+      </c>
+      <c r="BT33" s="18">
+        <v>2</v>
+      </c>
       <c r="BU33" s="18"/>
       <c r="BV33" s="18"/>
       <c r="BW33" s="18"/>
@@ -24119,7 +24135,7 @@
       </c>
       <c r="B68" s="7">
         <f t="shared" si="44"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C68" s="7"/>
       <c r="D68" s="7"/>
@@ -24177,7 +24193,9 @@
       <c r="BP68" s="18"/>
       <c r="BQ68" s="18"/>
       <c r="BR68" s="18"/>
-      <c r="BS68" s="18"/>
+      <c r="BS68" s="18">
+        <v>2</v>
+      </c>
       <c r="BT68" s="18"/>
       <c r="BU68" s="18"/>
       <c r="BV68" s="18"/>
@@ -26308,7 +26326,7 @@
       </c>
       <c r="B76" s="7">
         <f t="shared" si="45"/>
-        <v>31.5</v>
+        <v>33.5</v>
       </c>
       <c r="C76" s="7"/>
       <c r="D76" s="7"/>
@@ -26401,8 +26419,12 @@
       <c r="BR76" s="18">
         <v>3</v>
       </c>
-      <c r="BS76" s="18"/>
-      <c r="BT76" s="18"/>
+      <c r="BS76" s="18">
+        <v>1</v>
+      </c>
+      <c r="BT76" s="18">
+        <v>1</v>
+      </c>
       <c r="BU76" s="18"/>
       <c r="BV76" s="18"/>
       <c r="BW76" s="18"/>
@@ -26601,7 +26623,7 @@
       </c>
       <c r="B77" s="7">
         <f t="shared" si="45"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C77" s="7"/>
       <c r="D77" s="7"/>
@@ -26670,8 +26692,12 @@
       <c r="BP77" s="18"/>
       <c r="BQ77" s="18"/>
       <c r="BR77" s="18"/>
-      <c r="BS77" s="18"/>
-      <c r="BT77" s="18"/>
+      <c r="BS77" s="18">
+        <v>2</v>
+      </c>
+      <c r="BT77" s="18">
+        <v>1</v>
+      </c>
       <c r="BU77" s="18"/>
       <c r="BV77" s="18"/>
       <c r="BW77" s="18"/>
@@ -31122,6 +31148,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
     <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
@@ -31362,27 +31408,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{035973C1-EA40-447A-BB47-72CAA2093BEE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEFE62B7-6772-44D0-ACCE-A546E807D9BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B47248CD-DDBC-44C8-8FB9-07EFB28EB7F7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -31399,29 +31450,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{035973C1-EA40-447A-BB47-72CAA2093BEE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEFE62B7-6772-44D0-ACCE-A546E807D9BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Sync from OneDrive: DSafarik_2026TimeTracking.xlsx [2026-04-13 15:00 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ctbuh.sharepoint.com/sites/Staff/Shared Documents/Research/Time Tracking/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2491" documentId="8_{0FDB2C51-E576-4C63-8BE8-7A83A2F616A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BAB8FD7-37D2-4404-A060-4C7BFB7F9FE7}"/>
+  <xr:revisionPtr revIDLastSave="2500" documentId="8_{0FDB2C51-E576-4C63-8BE8-7A83A2F616A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F2ABCCA-4DFE-4EF7-992E-E98CF32284DD}"/>
   <bookViews>
-    <workbookView xWindow="28635" yWindow="-165" windowWidth="29130" windowHeight="17610" xr2:uid="{0C10F557-92E5-4EB6-9E48-62A8B86D346C}"/>
+    <workbookView minimized="1" xWindow="2110" yWindow="2340" windowWidth="13450" windowHeight="6680" xr2:uid="{0C10F557-92E5-4EB6-9E48-62A8B86D346C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tracking" sheetId="1" r:id="rId1"/>
@@ -1123,36 +1123,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA06A09C-89B1-4AA3-9EFC-90144A056127}">
   <dimension ref="A1:JC97"/>
-  <sheetFormatPr defaultColWidth="3.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="3.53515625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="37.85546875" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" customWidth="1"/>
-    <col min="3" max="7" width="3.5703125" customWidth="1"/>
-    <col min="8" max="8" width="3.42578125" customWidth="1"/>
-    <col min="9" max="23" width="3.5703125" customWidth="1"/>
-    <col min="24" max="24" width="3.5703125" style="27" customWidth="1"/>
-    <col min="25" max="43" width="3.5703125" customWidth="1"/>
-    <col min="44" max="44" width="3.5703125" style="27" customWidth="1"/>
-    <col min="45" max="65" width="3.5703125" customWidth="1"/>
-    <col min="66" max="66" width="3.5703125" style="27" customWidth="1"/>
-    <col min="67" max="87" width="3.5703125" customWidth="1"/>
-    <col min="88" max="88" width="3.5703125" style="27" customWidth="1"/>
-    <col min="89" max="108" width="3.5703125" customWidth="1"/>
-    <col min="109" max="109" width="3.5703125" style="27" customWidth="1"/>
-    <col min="110" max="130" width="3.5703125" customWidth="1"/>
-    <col min="131" max="131" width="3.5703125" style="27" customWidth="1"/>
-    <col min="132" max="153" width="3.5703125" customWidth="1"/>
-    <col min="154" max="154" width="3.5703125" style="27" customWidth="1"/>
-    <col min="155" max="174" width="3.5703125" customWidth="1"/>
-    <col min="175" max="175" width="3.5703125" style="27" customWidth="1"/>
-    <col min="176" max="188" width="3.5703125" customWidth="1"/>
-    <col min="197" max="197" width="3.5703125" style="27"/>
-    <col min="219" max="219" width="3.5703125" style="27"/>
-    <col min="240" max="240" width="3.5703125" style="27"/>
-    <col min="263" max="263" width="3.5703125" style="27"/>
+    <col min="1" max="1" width="37.84375" customWidth="1"/>
+    <col min="2" max="2" width="10.53515625" customWidth="1"/>
+    <col min="3" max="7" width="3.53515625" customWidth="1"/>
+    <col min="8" max="8" width="3.3828125" customWidth="1"/>
+    <col min="9" max="23" width="3.53515625" customWidth="1"/>
+    <col min="24" max="24" width="3.53515625" style="27" customWidth="1"/>
+    <col min="25" max="43" width="3.53515625" customWidth="1"/>
+    <col min="44" max="44" width="3.53515625" style="27" customWidth="1"/>
+    <col min="45" max="65" width="3.53515625" customWidth="1"/>
+    <col min="66" max="66" width="3.53515625" style="27" customWidth="1"/>
+    <col min="67" max="87" width="3.53515625" customWidth="1"/>
+    <col min="88" max="88" width="3.53515625" style="27" customWidth="1"/>
+    <col min="89" max="108" width="3.53515625" customWidth="1"/>
+    <col min="109" max="109" width="3.53515625" style="27" customWidth="1"/>
+    <col min="110" max="130" width="3.53515625" customWidth="1"/>
+    <col min="131" max="131" width="3.53515625" style="27" customWidth="1"/>
+    <col min="132" max="153" width="3.53515625" customWidth="1"/>
+    <col min="154" max="154" width="3.53515625" style="27" customWidth="1"/>
+    <col min="155" max="174" width="3.53515625" customWidth="1"/>
+    <col min="175" max="175" width="3.53515625" style="27" customWidth="1"/>
+    <col min="176" max="188" width="3.53515625" customWidth="1"/>
+    <col min="197" max="197" width="3.53515625" style="27"/>
+    <col min="219" max="219" width="3.53515625" style="27"/>
+    <col min="240" max="240" width="3.53515625" style="27"/>
+    <col min="263" max="263" width="3.53515625" style="27"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1441,11 +1441,11 @@
       </c>
       <c r="BU1" s="10">
         <f t="shared" ref="BU1:CD2" si="7">SUM(BU$7:BU$1048576)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BV1" s="10">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BW1" s="10">
         <f t="shared" si="7"/>
@@ -2204,7 +2204,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A2" s="4"/>
       <c r="B2" s="13" t="s">
         <v>2</v>
@@ -2491,11 +2491,11 @@
       </c>
       <c r="BU2" s="10">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BV2" s="10">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BW2" s="10">
         <f t="shared" si="7"/>
@@ -3254,7 +3254,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A3" s="4"/>
       <c r="B3" s="13" t="s">
         <v>3</v>
@@ -4304,7 +4304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:263" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:263" s="1" customFormat="1" ht="14.15" x14ac:dyDescent="0.4">
       <c r="B4" s="13" t="s">
         <v>4</v>
       </c>
@@ -5353,7 +5353,7 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="5" spans="1:263" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:263" s="1" customFormat="1" ht="14.15" x14ac:dyDescent="0.4">
       <c r="B5" s="13" t="s">
         <v>5</v>
       </c>
@@ -6141,7 +6141,7 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="6" spans="1:263" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:263" s="1" customFormat="1" ht="14.15" x14ac:dyDescent="0.4">
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
@@ -7193,13 +7193,13 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="7" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A7" s="8" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="11">
         <f>SUM(B8:B23)</f>
-        <v>167.25</v>
+        <v>169.25</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -7463,7 +7463,7 @@
       <c r="JB7" s="7"/>
       <c r="JC7" s="20"/>
     </row>
-    <row r="8" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
@@ -7733,7 +7733,7 @@
       <c r="JB8" s="7"/>
       <c r="JC8" s="20"/>
     </row>
-    <row r="9" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
@@ -8003,7 +8003,7 @@
       <c r="JB9" s="7"/>
       <c r="JC9" s="20"/>
     </row>
-    <row r="10" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A10" s="6" t="s">
         <v>11</v>
       </c>
@@ -8273,7 +8273,7 @@
       <c r="JB10" s="7"/>
       <c r="JC10" s="20"/>
     </row>
-    <row r="11" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A11" s="6" t="s">
         <v>72</v>
       </c>
@@ -8593,7 +8593,7 @@
       <c r="JB11" s="7"/>
       <c r="JC11" s="20"/>
     </row>
-    <row r="12" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A12" s="6" t="s">
         <v>73</v>
       </c>
@@ -8869,7 +8869,7 @@
       <c r="JB12" s="7"/>
       <c r="JC12" s="20"/>
     </row>
-    <row r="13" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A13" s="6" t="s">
         <v>74</v>
       </c>
@@ -9161,7 +9161,7 @@
       <c r="JB13" s="7"/>
       <c r="JC13" s="20"/>
     </row>
-    <row r="14" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A14" s="6" t="s">
         <v>75</v>
       </c>
@@ -9433,7 +9433,7 @@
       <c r="JB14" s="7"/>
       <c r="JC14" s="20"/>
     </row>
-    <row r="15" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A15" s="6" t="s">
         <v>12</v>
       </c>
@@ -9703,7 +9703,7 @@
       <c r="JB15" s="7"/>
       <c r="JC15" s="20"/>
     </row>
-    <row r="16" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A16" s="6" t="s">
         <v>13</v>
       </c>
@@ -9977,7 +9977,7 @@
       <c r="JB16" s="7"/>
       <c r="JC16" s="20"/>
     </row>
-    <row r="17" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A17" s="6" t="s">
         <v>14</v>
       </c>
@@ -10251,7 +10251,7 @@
       <c r="JB17" s="7"/>
       <c r="JC17" s="20"/>
     </row>
-    <row r="18" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A18" s="6" t="s">
         <v>15</v>
       </c>
@@ -10525,7 +10525,7 @@
       <c r="JB18" s="7"/>
       <c r="JC18" s="20"/>
     </row>
-    <row r="19" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A19" s="6" t="s">
         <v>16</v>
       </c>
@@ -10806,7 +10806,7 @@
       <c r="JB19" s="7"/>
       <c r="JC19" s="20"/>
     </row>
-    <row r="20" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A20" s="6" t="s">
         <v>17</v>
       </c>
@@ -11078,13 +11078,13 @@
       <c r="JB20" s="7"/>
       <c r="JC20" s="20"/>
     </row>
-    <row r="21" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A21" s="6" t="s">
         <v>18</v>
       </c>
       <c r="B21" s="7">
         <f t="shared" si="41"/>
-        <v>20.75</v>
+        <v>22.75</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
@@ -11199,7 +11199,9 @@
         <v>2</v>
       </c>
       <c r="BU21" s="18"/>
-      <c r="BV21" s="18"/>
+      <c r="BV21" s="18">
+        <v>2</v>
+      </c>
       <c r="BW21" s="18"/>
       <c r="BX21" s="18"/>
       <c r="BY21" s="18"/>
@@ -11390,7 +11392,7 @@
       <c r="JB21" s="7"/>
       <c r="JC21" s="20"/>
     </row>
-    <row r="22" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A22" s="6" t="s">
         <v>19</v>
       </c>
@@ -11660,7 +11662,7 @@
       <c r="JB22" s="7"/>
       <c r="JC22" s="20"/>
     </row>
-    <row r="23" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A23" s="6" t="s">
         <v>20</v>
       </c>
@@ -11969,7 +11971,7 @@
       <c r="JB23" s="7"/>
       <c r="JC23" s="20"/>
     </row>
-    <row r="24" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A24" s="8" t="s">
         <v>21</v>
       </c>
@@ -12236,7 +12238,7 @@
       <c r="JB24" s="7"/>
       <c r="JC24" s="20"/>
     </row>
-    <row r="25" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A25" s="6" t="s">
         <v>22</v>
       </c>
@@ -12506,7 +12508,7 @@
       <c r="JB25" s="7"/>
       <c r="JC25" s="20"/>
     </row>
-    <row r="26" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A26" s="6" t="s">
         <v>23</v>
       </c>
@@ -12776,7 +12778,7 @@
       <c r="JB26" s="7"/>
       <c r="JC26" s="20"/>
     </row>
-    <row r="27" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A27" s="6" t="s">
         <v>24</v>
       </c>
@@ -13046,7 +13048,7 @@
       <c r="JB27" s="7"/>
       <c r="JC27" s="20"/>
     </row>
-    <row r="28" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A28" s="6" t="s">
         <v>25</v>
       </c>
@@ -13316,7 +13318,7 @@
       <c r="JB28" s="7"/>
       <c r="JC28" s="20"/>
     </row>
-    <row r="29" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A29" s="6" t="s">
         <v>26</v>
       </c>
@@ -13586,7 +13588,7 @@
       <c r="JB29" s="7"/>
       <c r="JC29" s="20"/>
     </row>
-    <row r="30" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A30" s="8" t="s">
         <v>27</v>
       </c>
@@ -13853,13 +13855,13 @@
       <c r="JB30" s="7"/>
       <c r="JC30" s="20"/>
     </row>
-    <row r="31" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A31" s="6" t="s">
         <v>28</v>
       </c>
       <c r="B31" s="7">
         <f t="shared" ref="B31:B40" si="42">SUM($C31:$XFD31)</f>
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
@@ -14010,8 +14012,12 @@
       <c r="BT31" s="18">
         <v>2</v>
       </c>
-      <c r="BU31" s="18"/>
-      <c r="BV31" s="18"/>
+      <c r="BU31" s="18">
+        <v>2</v>
+      </c>
+      <c r="BV31" s="18">
+        <v>2</v>
+      </c>
       <c r="BW31" s="18"/>
       <c r="BX31" s="18"/>
       <c r="BY31" s="18"/>
@@ -14202,7 +14208,7 @@
       <c r="JB31" s="7"/>
       <c r="JC31" s="20"/>
     </row>
-    <row r="32" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A32" s="6" t="s">
         <v>29</v>
       </c>
@@ -14472,13 +14478,13 @@
       <c r="JB32" s="7"/>
       <c r="JC32" s="20"/>
     </row>
-    <row r="33" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A33" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="7">
         <f t="shared" si="42"/>
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
@@ -14598,8 +14604,12 @@
       <c r="BT33" s="18">
         <v>2</v>
       </c>
-      <c r="BU33" s="18"/>
-      <c r="BV33" s="18"/>
+      <c r="BU33" s="18">
+        <v>2</v>
+      </c>
+      <c r="BV33" s="18">
+        <v>2</v>
+      </c>
       <c r="BW33" s="18"/>
       <c r="BX33" s="18"/>
       <c r="BY33" s="18"/>
@@ -14790,7 +14800,7 @@
       <c r="JB33" s="7"/>
       <c r="JC33" s="20"/>
     </row>
-    <row r="34" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A34" s="6" t="s">
         <v>31</v>
       </c>
@@ -15060,7 +15070,7 @@
       <c r="JB34" s="7"/>
       <c r="JC34" s="20"/>
     </row>
-    <row r="35" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A35" s="6" t="s">
         <v>32</v>
       </c>
@@ -15332,7 +15342,7 @@
       <c r="JB35" s="7"/>
       <c r="JC35" s="20"/>
     </row>
-    <row r="36" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A36" s="6" t="s">
         <v>33</v>
       </c>
@@ -15602,7 +15612,7 @@
       <c r="JB36" s="7"/>
       <c r="JC36" s="20"/>
     </row>
-    <row r="37" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A37" s="6" t="s">
         <v>34</v>
       </c>
@@ -15872,7 +15882,7 @@
       <c r="JB37" s="7"/>
       <c r="JC37" s="20"/>
     </row>
-    <row r="38" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A38" s="6" t="s">
         <v>35</v>
       </c>
@@ -16142,7 +16152,7 @@
       <c r="JB38" s="7"/>
       <c r="JC38" s="20"/>
     </row>
-    <row r="39" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A39" s="6" t="s">
         <v>36</v>
       </c>
@@ -16412,7 +16422,7 @@
       <c r="JB39" s="7"/>
       <c r="JC39" s="20"/>
     </row>
-    <row r="40" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A40" s="6" t="s">
         <v>37</v>
       </c>
@@ -16684,7 +16694,7 @@
       <c r="JB40" s="7"/>
       <c r="JC40" s="20"/>
     </row>
-    <row r="41" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A41" s="8" t="s">
         <v>38</v>
       </c>
@@ -16951,7 +16961,7 @@
       <c r="JB41" s="7"/>
       <c r="JC41" s="20"/>
     </row>
-    <row r="42" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A42" s="6" t="s">
         <v>39</v>
       </c>
@@ -17221,7 +17231,7 @@
       <c r="JB42" s="7"/>
       <c r="JC42" s="20"/>
     </row>
-    <row r="43" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A43" s="6" t="s">
         <v>76</v>
       </c>
@@ -17491,7 +17501,7 @@
       <c r="JB43" s="7"/>
       <c r="JC43" s="20"/>
     </row>
-    <row r="44" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A44" s="6" t="s">
         <v>77</v>
       </c>
@@ -17761,7 +17771,7 @@
       <c r="JB44" s="7"/>
       <c r="JC44" s="20"/>
     </row>
-    <row r="45" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A45" s="6" t="s">
         <v>78</v>
       </c>
@@ -18031,7 +18041,7 @@
       <c r="JB45" s="7"/>
       <c r="JC45" s="20"/>
     </row>
-    <row r="46" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A46" s="6" t="s">
         <v>40</v>
       </c>
@@ -18307,7 +18317,7 @@
       <c r="JB46" s="7"/>
       <c r="JC46" s="20"/>
     </row>
-    <row r="47" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A47" s="6" t="s">
         <v>41</v>
       </c>
@@ -18577,7 +18587,7 @@
       <c r="JB47" s="7"/>
       <c r="JC47" s="20"/>
     </row>
-    <row r="48" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A48" s="6" t="s">
         <v>42</v>
       </c>
@@ -18847,7 +18857,7 @@
       <c r="JB48" s="7"/>
       <c r="JC48" s="20"/>
     </row>
-    <row r="49" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A49" s="6" t="s">
         <v>43</v>
       </c>
@@ -19117,7 +19127,7 @@
       <c r="JB49" s="7"/>
       <c r="JC49" s="20"/>
     </row>
-    <row r="50" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A50" s="6" t="s">
         <v>44</v>
       </c>
@@ -19389,7 +19399,7 @@
       <c r="JB50" s="7"/>
       <c r="JC50" s="20"/>
     </row>
-    <row r="51" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A51" s="8" t="s">
         <v>45</v>
       </c>
@@ -19656,7 +19666,7 @@
       <c r="JB51" s="7"/>
       <c r="JC51" s="20"/>
     </row>
-    <row r="52" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A52" s="6" t="s">
         <v>46</v>
       </c>
@@ -19926,7 +19936,7 @@
       <c r="JB52" s="7"/>
       <c r="JC52" s="20"/>
     </row>
-    <row r="53" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A53" s="6" t="s">
         <v>47</v>
       </c>
@@ -20200,7 +20210,7 @@
       <c r="JB53" s="7"/>
       <c r="JC53" s="20"/>
     </row>
-    <row r="54" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A54" s="6" t="s">
         <v>48</v>
       </c>
@@ -20482,7 +20492,7 @@
       <c r="JB54" s="7"/>
       <c r="JC54" s="20"/>
     </row>
-    <row r="55" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A55" s="8" t="s">
         <v>49</v>
       </c>
@@ -20749,7 +20759,7 @@
       <c r="JB55" s="7"/>
       <c r="JC55" s="20"/>
     </row>
-    <row r="56" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A56" s="6" t="s">
         <v>50</v>
       </c>
@@ -21019,7 +21029,7 @@
       <c r="JB56" s="7"/>
       <c r="JC56" s="20"/>
     </row>
-    <row r="57" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A57" s="6" t="s">
         <v>51</v>
       </c>
@@ -21289,7 +21299,7 @@
       <c r="JB57" s="7"/>
       <c r="JC57" s="20"/>
     </row>
-    <row r="58" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A58" s="6" t="s">
         <v>52</v>
       </c>
@@ -21559,7 +21569,7 @@
       <c r="JB58" s="7"/>
       <c r="JC58" s="20"/>
     </row>
-    <row r="59" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A59" s="6" t="s">
         <v>53</v>
       </c>
@@ -21829,7 +21839,7 @@
       <c r="JB59" s="7"/>
       <c r="JC59" s="20"/>
     </row>
-    <row r="60" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A60" s="6" t="s">
         <v>54</v>
       </c>
@@ -22099,7 +22109,7 @@
       <c r="JB60" s="7"/>
       <c r="JC60" s="20"/>
     </row>
-    <row r="61" spans="1:263" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:263" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A61" s="8" t="s">
         <v>55</v>
       </c>
@@ -22366,7 +22376,7 @@
       <c r="JB61" s="7"/>
       <c r="JC61" s="20"/>
     </row>
-    <row r="62" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A62" s="6" t="s">
         <v>56</v>
       </c>
@@ -22638,7 +22648,7 @@
       <c r="JB62" s="7"/>
       <c r="JC62" s="20"/>
     </row>
-    <row r="63" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A63" s="6" t="s">
         <v>57</v>
       </c>
@@ -23005,7 +23015,7 @@
       <c r="JB63" s="7"/>
       <c r="JC63" s="20"/>
     </row>
-    <row r="64" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A64" s="6" t="s">
         <v>58</v>
       </c>
@@ -23280,7 +23290,7 @@
       <c r="JB64" s="7"/>
       <c r="JC64" s="20"/>
     </row>
-    <row r="65" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A65" s="6" t="s">
         <v>59</v>
       </c>
@@ -23549,7 +23559,7 @@
       <c r="JB65" s="7"/>
       <c r="JC65" s="20"/>
     </row>
-    <row r="66" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A66" s="6" t="s">
         <v>79</v>
       </c>
@@ -23858,7 +23868,7 @@
       <c r="JB66" s="7"/>
       <c r="JC66" s="20"/>
     </row>
-    <row r="67" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A67" s="6" t="s">
         <v>80</v>
       </c>
@@ -24129,13 +24139,13 @@
       <c r="JB67" s="7"/>
       <c r="JC67" s="20"/>
     </row>
-    <row r="68" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A68" s="6" t="s">
         <v>82</v>
       </c>
       <c r="B68" s="7">
         <f t="shared" si="44"/>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C68" s="7"/>
       <c r="D68" s="7"/>
@@ -24197,8 +24207,12 @@
         <v>2</v>
       </c>
       <c r="BT68" s="18"/>
-      <c r="BU68" s="18"/>
-      <c r="BV68" s="18"/>
+      <c r="BU68" s="18">
+        <v>2</v>
+      </c>
+      <c r="BV68" s="18">
+        <v>2</v>
+      </c>
       <c r="BW68" s="18"/>
       <c r="BX68" s="18"/>
       <c r="BY68" s="18"/>
@@ -24389,7 +24403,7 @@
       <c r="JB68" s="7"/>
       <c r="JC68" s="20"/>
     </row>
-    <row r="69" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A69" s="6" t="s">
         <v>81</v>
       </c>
@@ -24658,7 +24672,7 @@
       <c r="JB69" s="7"/>
       <c r="JC69" s="20"/>
     </row>
-    <row r="70" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A70" s="8" t="s">
         <v>60</v>
       </c>
@@ -24924,7 +24938,7 @@
       <c r="JB70" s="7"/>
       <c r="JC70" s="20"/>
     </row>
-    <row r="71" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A71" s="6" t="s">
         <v>61</v>
       </c>
@@ -25197,7 +25211,7 @@
       <c r="JB71" s="7"/>
       <c r="JC71" s="20"/>
     </row>
-    <row r="72" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A72" s="6" t="s">
         <v>62</v>
       </c>
@@ -25466,7 +25480,7 @@
       <c r="JB72" s="7"/>
       <c r="JC72" s="20"/>
     </row>
-    <row r="73" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A73" s="6" t="s">
         <v>63</v>
       </c>
@@ -25735,7 +25749,7 @@
       <c r="JB73" s="7"/>
       <c r="JC73" s="20"/>
     </row>
-    <row r="74" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A74" s="8" t="s">
         <v>64</v>
       </c>
@@ -26001,7 +26015,7 @@
       <c r="JB74" s="7"/>
       <c r="JC74" s="20"/>
     </row>
-    <row r="75" spans="1:263" s="12" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:263" s="12" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
         <v>83</v>
       </c>
@@ -26320,7 +26334,7 @@
       <c r="JB75" s="7"/>
       <c r="JC75" s="20"/>
     </row>
-    <row r="76" spans="1:263" s="12" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:263" s="12" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="6" t="s">
         <v>84</v>
       </c>
@@ -26617,13 +26631,13 @@
       <c r="JB76" s="7"/>
       <c r="JC76" s="20"/>
     </row>
-    <row r="77" spans="1:263" s="12" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:263" s="12" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
         <v>85</v>
       </c>
       <c r="B77" s="7">
         <f t="shared" si="45"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C77" s="7"/>
       <c r="D77" s="7"/>
@@ -26698,7 +26712,9 @@
       <c r="BT77" s="18">
         <v>1</v>
       </c>
-      <c r="BU77" s="18"/>
+      <c r="BU77" s="18">
+        <v>1</v>
+      </c>
       <c r="BV77" s="18"/>
       <c r="BW77" s="18"/>
       <c r="BX77" s="18"/>
@@ -26890,7 +26906,7 @@
       <c r="JB77" s="7"/>
       <c r="JC77" s="20"/>
     </row>
-    <row r="78" spans="1:263" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:263" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A78" s="6" t="s">
         <v>65</v>
       </c>
@@ -27162,7 +27178,7 @@
       <c r="JB78" s="7"/>
       <c r="JC78" s="20"/>
     </row>
-    <row r="79" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A79" s="6" t="s">
         <v>66</v>
       </c>
@@ -27432,7 +27448,7 @@
       <c r="JB79" s="7"/>
       <c r="JC79" s="20"/>
     </row>
-    <row r="80" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A80" s="6" t="s">
         <v>67</v>
       </c>
@@ -27724,7 +27740,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="81" spans="1:263" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:263" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A81" s="6" t="s">
         <v>68</v>
       </c>
@@ -28004,7 +28020,7 @@
       <c r="JB81" s="7"/>
       <c r="JC81" s="20"/>
     </row>
-    <row r="82" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A82" s="6" t="s">
         <v>69</v>
       </c>
@@ -28278,13 +28294,13 @@
       <c r="JB82" s="7"/>
       <c r="JC82" s="20"/>
     </row>
-    <row r="83" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A83" s="9" t="s">
         <v>70</v>
       </c>
       <c r="B83" s="7">
         <f t="shared" si="46"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C83" s="7"/>
       <c r="D83" s="7"/>
@@ -28360,7 +28376,9 @@
       <c r="BR83" s="18"/>
       <c r="BS83" s="18"/>
       <c r="BT83" s="18"/>
-      <c r="BU83" s="18"/>
+      <c r="BU83" s="18">
+        <v>1</v>
+      </c>
       <c r="BV83" s="18"/>
       <c r="BW83" s="18"/>
       <c r="BX83" s="18"/>
@@ -28552,7 +28570,7 @@
       <c r="JB83" s="7"/>
       <c r="JC83" s="20"/>
     </row>
-    <row r="84" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:263" x14ac:dyDescent="0.4">
       <c r="A84" s="6" t="s">
         <v>71</v>
       </c>
@@ -28822,7 +28840,7 @@
       <c r="JB84" s="7"/>
       <c r="JC84" s="20"/>
     </row>
-    <row r="85" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:263" x14ac:dyDescent="0.4">
       <c r="B85" s="7"/>
       <c r="E85" s="25"/>
       <c r="F85" s="25"/>
@@ -29010,7 +29028,7 @@
       <c r="GF85" s="25"/>
       <c r="GG85" s="25"/>
     </row>
-    <row r="86" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:263" x14ac:dyDescent="0.4">
       <c r="B86" s="24"/>
       <c r="E86" s="25"/>
       <c r="F86" s="25"/>
@@ -29198,7 +29216,7 @@
       <c r="GF86" s="25"/>
       <c r="GG86" s="25"/>
     </row>
-    <row r="87" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:263" x14ac:dyDescent="0.4">
       <c r="B87" s="7"/>
       <c r="E87" s="25"/>
       <c r="F87" s="25"/>
@@ -29386,7 +29404,7 @@
       <c r="GF87" s="25"/>
       <c r="GG87" s="25"/>
     </row>
-    <row r="88" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:263" x14ac:dyDescent="0.4">
       <c r="B88" s="7"/>
       <c r="E88" s="25"/>
       <c r="F88" s="25"/>
@@ -29574,7 +29592,7 @@
       <c r="GF88" s="25"/>
       <c r="GG88" s="25"/>
     </row>
-    <row r="89" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:263" x14ac:dyDescent="0.4">
       <c r="B89" s="7"/>
       <c r="E89" s="25"/>
       <c r="F89" s="25"/>
@@ -29762,7 +29780,7 @@
       <c r="GF89" s="25"/>
       <c r="GG89" s="25"/>
     </row>
-    <row r="90" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:263" x14ac:dyDescent="0.4">
       <c r="B90" s="7"/>
       <c r="E90" s="25"/>
       <c r="F90" s="25"/>
@@ -29950,7 +29968,7 @@
       <c r="GF90" s="25"/>
       <c r="GG90" s="25"/>
     </row>
-    <row r="91" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:263" x14ac:dyDescent="0.4">
       <c r="B91" s="7"/>
       <c r="E91" s="25"/>
       <c r="F91" s="25"/>
@@ -30138,7 +30156,7 @@
       <c r="GF91" s="25"/>
       <c r="GG91" s="25"/>
     </row>
-    <row r="92" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:263" x14ac:dyDescent="0.4">
       <c r="B92" s="7"/>
       <c r="E92" s="25"/>
       <c r="F92" s="25"/>
@@ -30326,7 +30344,7 @@
       <c r="GF92" s="25"/>
       <c r="GG92" s="25"/>
     </row>
-    <row r="93" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:263" x14ac:dyDescent="0.4">
       <c r="B93" s="7"/>
       <c r="E93" s="25"/>
       <c r="F93" s="25"/>
@@ -30514,7 +30532,7 @@
       <c r="GF93" s="25"/>
       <c r="GG93" s="25"/>
     </row>
-    <row r="94" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:263" x14ac:dyDescent="0.4">
       <c r="B94" s="7"/>
       <c r="E94" s="25"/>
       <c r="F94" s="25"/>
@@ -30702,7 +30720,7 @@
       <c r="GF94" s="25"/>
       <c r="GG94" s="25"/>
     </row>
-    <row r="95" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:263" x14ac:dyDescent="0.4">
       <c r="B95" s="7"/>
       <c r="E95" s="25"/>
       <c r="F95" s="25"/>
@@ -30890,7 +30908,7 @@
       <c r="GF95" s="25"/>
       <c r="GG95" s="25"/>
     </row>
-    <row r="96" spans="1:263" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:263" x14ac:dyDescent="0.4">
       <c r="B96" s="7"/>
       <c r="E96" s="25"/>
       <c r="F96" s="25"/>
@@ -31078,7 +31096,7 @@
       <c r="GF96" s="25"/>
       <c r="GG96" s="25"/>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B97" s="7"/>
     </row>
   </sheetData>
@@ -31148,26 +31166,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
     <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
@@ -31408,32 +31406,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{035973C1-EA40-447A-BB47-72CAA2093BEE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEFE62B7-6772-44D0-ACCE-A546E807D9BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B47248CD-DDBC-44C8-8FB9-07EFB28EB7F7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -31450,4 +31443,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEFE62B7-6772-44D0-ACCE-A546E807D9BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{035973C1-EA40-447A-BB47-72CAA2093BEE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Sync from OneDrive: DSafarik_2026TimeTracking.xlsx [2026-04-13 17:00 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ctbuh.sharepoint.com/sites/Staff/Shared Documents/Research/Time Tracking/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2500" documentId="8_{0FDB2C51-E576-4C63-8BE8-7A83A2F616A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F2ABCCA-4DFE-4EF7-992E-E98CF32284DD}"/>
+  <xr:revisionPtr revIDLastSave="2504" documentId="8_{0FDB2C51-E576-4C63-8BE8-7A83A2F616A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21C27188-B84B-4522-AE40-2D8DBCE00B59}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2110" yWindow="2340" windowWidth="13450" windowHeight="6680" xr2:uid="{0C10F557-92E5-4EB6-9E48-62A8B86D346C}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{0C10F557-92E5-4EB6-9E48-62A8B86D346C}"/>
   </bookViews>
   <sheets>
     <sheet name="Tracking" sheetId="1" r:id="rId1"/>
@@ -1123,36 +1123,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA06A09C-89B1-4AA3-9EFC-90144A056127}">
   <dimension ref="A1:JC97"/>
-  <sheetFormatPr defaultColWidth="3.53515625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="3.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.84375" customWidth="1"/>
-    <col min="2" max="2" width="10.53515625" customWidth="1"/>
-    <col min="3" max="7" width="3.53515625" customWidth="1"/>
-    <col min="8" max="8" width="3.3828125" customWidth="1"/>
-    <col min="9" max="23" width="3.53515625" customWidth="1"/>
-    <col min="24" max="24" width="3.53515625" style="27" customWidth="1"/>
-    <col min="25" max="43" width="3.53515625" customWidth="1"/>
-    <col min="44" max="44" width="3.53515625" style="27" customWidth="1"/>
-    <col min="45" max="65" width="3.53515625" customWidth="1"/>
-    <col min="66" max="66" width="3.53515625" style="27" customWidth="1"/>
-    <col min="67" max="87" width="3.53515625" customWidth="1"/>
-    <col min="88" max="88" width="3.53515625" style="27" customWidth="1"/>
-    <col min="89" max="108" width="3.53515625" customWidth="1"/>
-    <col min="109" max="109" width="3.53515625" style="27" customWidth="1"/>
-    <col min="110" max="130" width="3.53515625" customWidth="1"/>
-    <col min="131" max="131" width="3.53515625" style="27" customWidth="1"/>
-    <col min="132" max="153" width="3.53515625" customWidth="1"/>
-    <col min="154" max="154" width="3.53515625" style="27" customWidth="1"/>
-    <col min="155" max="174" width="3.53515625" customWidth="1"/>
-    <col min="175" max="175" width="3.53515625" style="27" customWidth="1"/>
-    <col min="176" max="188" width="3.53515625" customWidth="1"/>
-    <col min="197" max="197" width="3.53515625" style="27"/>
-    <col min="219" max="219" width="3.53515625" style="27"/>
-    <col min="240" max="240" width="3.53515625" style="27"/>
-    <col min="263" max="263" width="3.53515625" style="27"/>
+    <col min="1" max="1" width="37.85546875" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" customWidth="1"/>
+    <col min="3" max="7" width="3.5703125" customWidth="1"/>
+    <col min="8" max="8" width="3.42578125" customWidth="1"/>
+    <col min="9" max="23" width="3.5703125" customWidth="1"/>
+    <col min="24" max="24" width="3.5703125" style="27" customWidth="1"/>
+    <col min="25" max="43" width="3.5703125" customWidth="1"/>
+    <col min="44" max="44" width="3.5703125" style="27" customWidth="1"/>
+    <col min="45" max="65" width="3.5703125" customWidth="1"/>
+    <col min="66" max="66" width="3.5703125" style="27" customWidth="1"/>
+    <col min="67" max="87" width="3.5703125" customWidth="1"/>
+    <col min="88" max="88" width="3.5703125" style="27" customWidth="1"/>
+    <col min="89" max="108" width="3.5703125" customWidth="1"/>
+    <col min="109" max="109" width="3.5703125" style="27" customWidth="1"/>
+    <col min="110" max="130" width="3.5703125" customWidth="1"/>
+    <col min="131" max="131" width="3.5703125" style="27" customWidth="1"/>
+    <col min="132" max="153" width="3.5703125" customWidth="1"/>
+    <col min="154" max="154" width="3.5703125" style="27" customWidth="1"/>
+    <col min="155" max="174" width="3.5703125" customWidth="1"/>
+    <col min="175" max="175" width="3.5703125" style="27" customWidth="1"/>
+    <col min="176" max="188" width="3.5703125" customWidth="1"/>
+    <col min="197" max="197" width="3.5703125" style="27"/>
+    <col min="219" max="219" width="3.5703125" style="27"/>
+    <col min="240" max="240" width="3.5703125" style="27"/>
+    <col min="263" max="263" width="3.5703125" style="27"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="BW1" s="10">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="BX1" s="10">
         <f t="shared" si="7"/>
@@ -2204,7 +2204,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A2" s="4"/>
       <c r="B2" s="13" t="s">
         <v>2</v>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="BW2" s="10">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="BX2" s="10">
         <f t="shared" si="7"/>
@@ -3254,7 +3254,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A3" s="4"/>
       <c r="B3" s="13" t="s">
         <v>3</v>
@@ -4304,7 +4304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:263" s="1" customFormat="1" ht="14.15" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:263" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B4" s="13" t="s">
         <v>4</v>
       </c>
@@ -5353,7 +5353,7 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="5" spans="1:263" s="1" customFormat="1" ht="14.15" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:263" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
       <c r="B5" s="13" t="s">
         <v>5</v>
       </c>
@@ -6141,7 +6141,7 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="6" spans="1:263" s="1" customFormat="1" ht="14.15" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:263" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
@@ -7193,13 +7193,13 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="7" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>8</v>
       </c>
       <c r="B7" s="11">
         <f>SUM(B8:B23)</f>
-        <v>169.25</v>
+        <v>170.25</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -7463,7 +7463,7 @@
       <c r="JB7" s="7"/>
       <c r="JC7" s="20"/>
     </row>
-    <row r="8" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
@@ -7733,7 +7733,7 @@
       <c r="JB8" s="7"/>
       <c r="JC8" s="20"/>
     </row>
-    <row r="9" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
@@ -8003,7 +8003,7 @@
       <c r="JB9" s="7"/>
       <c r="JC9" s="20"/>
     </row>
-    <row r="10" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>11</v>
       </c>
@@ -8273,13 +8273,13 @@
       <c r="JB10" s="7"/>
       <c r="JC10" s="20"/>
     </row>
-    <row r="11" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>72</v>
       </c>
       <c r="B11" s="7">
         <f t="shared" si="41"/>
-        <v>32.5</v>
+        <v>33.5</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -8403,7 +8403,9 @@
       <c r="BT11" s="18"/>
       <c r="BU11" s="18"/>
       <c r="BV11" s="18"/>
-      <c r="BW11" s="18"/>
+      <c r="BW11" s="18">
+        <v>1</v>
+      </c>
       <c r="BX11" s="18"/>
       <c r="BY11" s="18"/>
       <c r="BZ11" s="18"/>
@@ -8593,7 +8595,7 @@
       <c r="JB11" s="7"/>
       <c r="JC11" s="20"/>
     </row>
-    <row r="12" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>73</v>
       </c>
@@ -8869,7 +8871,7 @@
       <c r="JB12" s="7"/>
       <c r="JC12" s="20"/>
     </row>
-    <row r="13" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>74</v>
       </c>
@@ -9161,7 +9163,7 @@
       <c r="JB13" s="7"/>
       <c r="JC13" s="20"/>
     </row>
-    <row r="14" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>75</v>
       </c>
@@ -9433,7 +9435,7 @@
       <c r="JB14" s="7"/>
       <c r="JC14" s="20"/>
     </row>
-    <row r="15" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>12</v>
       </c>
@@ -9703,7 +9705,7 @@
       <c r="JB15" s="7"/>
       <c r="JC15" s="20"/>
     </row>
-    <row r="16" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>13</v>
       </c>
@@ -9977,7 +9979,7 @@
       <c r="JB16" s="7"/>
       <c r="JC16" s="20"/>
     </row>
-    <row r="17" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>14</v>
       </c>
@@ -10251,7 +10253,7 @@
       <c r="JB17" s="7"/>
       <c r="JC17" s="20"/>
     </row>
-    <row r="18" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>15</v>
       </c>
@@ -10525,7 +10527,7 @@
       <c r="JB18" s="7"/>
       <c r="JC18" s="20"/>
     </row>
-    <row r="19" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>16</v>
       </c>
@@ -10806,7 +10808,7 @@
       <c r="JB19" s="7"/>
       <c r="JC19" s="20"/>
     </row>
-    <row r="20" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>17</v>
       </c>
@@ -11078,7 +11080,7 @@
       <c r="JB20" s="7"/>
       <c r="JC20" s="20"/>
     </row>
-    <row r="21" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>18</v>
       </c>
@@ -11392,7 +11394,7 @@
       <c r="JB21" s="7"/>
       <c r="JC21" s="20"/>
     </row>
-    <row r="22" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>19</v>
       </c>
@@ -11662,7 +11664,7 @@
       <c r="JB22" s="7"/>
       <c r="JC22" s="20"/>
     </row>
-    <row r="23" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>20</v>
       </c>
@@ -11971,7 +11973,7 @@
       <c r="JB23" s="7"/>
       <c r="JC23" s="20"/>
     </row>
-    <row r="24" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
         <v>21</v>
       </c>
@@ -12238,7 +12240,7 @@
       <c r="JB24" s="7"/>
       <c r="JC24" s="20"/>
     </row>
-    <row r="25" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>22</v>
       </c>
@@ -12508,7 +12510,7 @@
       <c r="JB25" s="7"/>
       <c r="JC25" s="20"/>
     </row>
-    <row r="26" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>23</v>
       </c>
@@ -12778,7 +12780,7 @@
       <c r="JB26" s="7"/>
       <c r="JC26" s="20"/>
     </row>
-    <row r="27" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>24</v>
       </c>
@@ -13048,7 +13050,7 @@
       <c r="JB27" s="7"/>
       <c r="JC27" s="20"/>
     </row>
-    <row r="28" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>25</v>
       </c>
@@ -13318,7 +13320,7 @@
       <c r="JB28" s="7"/>
       <c r="JC28" s="20"/>
     </row>
-    <row r="29" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>26</v>
       </c>
@@ -13588,7 +13590,7 @@
       <c r="JB29" s="7"/>
       <c r="JC29" s="20"/>
     </row>
-    <row r="30" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>27</v>
       </c>
@@ -13855,13 +13857,13 @@
       <c r="JB30" s="7"/>
       <c r="JC30" s="20"/>
     </row>
-    <row r="31" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>28</v>
       </c>
       <c r="B31" s="7">
         <f t="shared" ref="B31:B40" si="42">SUM($C31:$XFD31)</f>
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
@@ -14018,7 +14020,9 @@
       <c r="BV31" s="18">
         <v>2</v>
       </c>
-      <c r="BW31" s="18"/>
+      <c r="BW31" s="18">
+        <v>2</v>
+      </c>
       <c r="BX31" s="18"/>
       <c r="BY31" s="18"/>
       <c r="BZ31" s="18"/>
@@ -14208,7 +14212,7 @@
       <c r="JB31" s="7"/>
       <c r="JC31" s="20"/>
     </row>
-    <row r="32" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>29</v>
       </c>
@@ -14478,13 +14482,13 @@
       <c r="JB32" s="7"/>
       <c r="JC32" s="20"/>
     </row>
-    <row r="33" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B33" s="7">
         <f t="shared" si="42"/>
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
@@ -14610,7 +14614,9 @@
       <c r="BV33" s="18">
         <v>2</v>
       </c>
-      <c r="BW33" s="18"/>
+      <c r="BW33" s="18">
+        <v>1</v>
+      </c>
       <c r="BX33" s="18"/>
       <c r="BY33" s="18"/>
       <c r="BZ33" s="18"/>
@@ -14800,7 +14806,7 @@
       <c r="JB33" s="7"/>
       <c r="JC33" s="20"/>
     </row>
-    <row r="34" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>31</v>
       </c>
@@ -15070,7 +15076,7 @@
       <c r="JB34" s="7"/>
       <c r="JC34" s="20"/>
     </row>
-    <row r="35" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>32</v>
       </c>
@@ -15342,7 +15348,7 @@
       <c r="JB35" s="7"/>
       <c r="JC35" s="20"/>
     </row>
-    <row r="36" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>33</v>
       </c>
@@ -15612,7 +15618,7 @@
       <c r="JB36" s="7"/>
       <c r="JC36" s="20"/>
     </row>
-    <row r="37" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>34</v>
       </c>
@@ -15882,7 +15888,7 @@
       <c r="JB37" s="7"/>
       <c r="JC37" s="20"/>
     </row>
-    <row r="38" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>35</v>
       </c>
@@ -16152,7 +16158,7 @@
       <c r="JB38" s="7"/>
       <c r="JC38" s="20"/>
     </row>
-    <row r="39" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>36</v>
       </c>
@@ -16422,7 +16428,7 @@
       <c r="JB39" s="7"/>
       <c r="JC39" s="20"/>
     </row>
-    <row r="40" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>37</v>
       </c>
@@ -16694,7 +16700,7 @@
       <c r="JB40" s="7"/>
       <c r="JC40" s="20"/>
     </row>
-    <row r="41" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
         <v>38</v>
       </c>
@@ -16961,7 +16967,7 @@
       <c r="JB41" s="7"/>
       <c r="JC41" s="20"/>
     </row>
-    <row r="42" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>39</v>
       </c>
@@ -17231,7 +17237,7 @@
       <c r="JB42" s="7"/>
       <c r="JC42" s="20"/>
     </row>
-    <row r="43" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>76</v>
       </c>
@@ -17501,7 +17507,7 @@
       <c r="JB43" s="7"/>
       <c r="JC43" s="20"/>
     </row>
-    <row r="44" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A44" s="6" t="s">
         <v>77</v>
       </c>
@@ -17771,7 +17777,7 @@
       <c r="JB44" s="7"/>
       <c r="JC44" s="20"/>
     </row>
-    <row r="45" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>78</v>
       </c>
@@ -18041,7 +18047,7 @@
       <c r="JB45" s="7"/>
       <c r="JC45" s="20"/>
     </row>
-    <row r="46" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>40</v>
       </c>
@@ -18317,7 +18323,7 @@
       <c r="JB46" s="7"/>
       <c r="JC46" s="20"/>
     </row>
-    <row r="47" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>41</v>
       </c>
@@ -18587,7 +18593,7 @@
       <c r="JB47" s="7"/>
       <c r="JC47" s="20"/>
     </row>
-    <row r="48" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>42</v>
       </c>
@@ -18857,7 +18863,7 @@
       <c r="JB48" s="7"/>
       <c r="JC48" s="20"/>
     </row>
-    <row r="49" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>43</v>
       </c>
@@ -19127,7 +19133,7 @@
       <c r="JB49" s="7"/>
       <c r="JC49" s="20"/>
     </row>
-    <row r="50" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>44</v>
       </c>
@@ -19399,7 +19405,7 @@
       <c r="JB50" s="7"/>
       <c r="JC50" s="20"/>
     </row>
-    <row r="51" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
         <v>45</v>
       </c>
@@ -19666,7 +19672,7 @@
       <c r="JB51" s="7"/>
       <c r="JC51" s="20"/>
     </row>
-    <row r="52" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>46</v>
       </c>
@@ -19936,7 +19942,7 @@
       <c r="JB52" s="7"/>
       <c r="JC52" s="20"/>
     </row>
-    <row r="53" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>47</v>
       </c>
@@ -20210,7 +20216,7 @@
       <c r="JB53" s="7"/>
       <c r="JC53" s="20"/>
     </row>
-    <row r="54" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>48</v>
       </c>
@@ -20492,7 +20498,7 @@
       <c r="JB54" s="7"/>
       <c r="JC54" s="20"/>
     </row>
-    <row r="55" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
         <v>49</v>
       </c>
@@ -20759,7 +20765,7 @@
       <c r="JB55" s="7"/>
       <c r="JC55" s="20"/>
     </row>
-    <row r="56" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
         <v>50</v>
       </c>
@@ -21029,7 +21035,7 @@
       <c r="JB56" s="7"/>
       <c r="JC56" s="20"/>
     </row>
-    <row r="57" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>51</v>
       </c>
@@ -21299,7 +21305,7 @@
       <c r="JB57" s="7"/>
       <c r="JC57" s="20"/>
     </row>
-    <row r="58" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
         <v>52</v>
       </c>
@@ -21569,7 +21575,7 @@
       <c r="JB58" s="7"/>
       <c r="JC58" s="20"/>
     </row>
-    <row r="59" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>53</v>
       </c>
@@ -21839,7 +21845,7 @@
       <c r="JB59" s="7"/>
       <c r="JC59" s="20"/>
     </row>
-    <row r="60" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>54</v>
       </c>
@@ -22109,7 +22115,7 @@
       <c r="JB60" s="7"/>
       <c r="JC60" s="20"/>
     </row>
-    <row r="61" spans="1:263" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:263" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
         <v>55</v>
       </c>
@@ -22376,7 +22382,7 @@
       <c r="JB61" s="7"/>
       <c r="JC61" s="20"/>
     </row>
-    <row r="62" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>56</v>
       </c>
@@ -22648,7 +22654,7 @@
       <c r="JB62" s="7"/>
       <c r="JC62" s="20"/>
     </row>
-    <row r="63" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>57</v>
       </c>
@@ -23015,7 +23021,7 @@
       <c r="JB63" s="7"/>
       <c r="JC63" s="20"/>
     </row>
-    <row r="64" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>58</v>
       </c>
@@ -23290,7 +23296,7 @@
       <c r="JB64" s="7"/>
       <c r="JC64" s="20"/>
     </row>
-    <row r="65" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>59</v>
       </c>
@@ -23559,7 +23565,7 @@
       <c r="JB65" s="7"/>
       <c r="JC65" s="20"/>
     </row>
-    <row r="66" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>79</v>
       </c>
@@ -23868,7 +23874,7 @@
       <c r="JB66" s="7"/>
       <c r="JC66" s="20"/>
     </row>
-    <row r="67" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>80</v>
       </c>
@@ -24139,13 +24145,13 @@
       <c r="JB67" s="7"/>
       <c r="JC67" s="20"/>
     </row>
-    <row r="68" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>82</v>
       </c>
       <c r="B68" s="7">
         <f t="shared" si="44"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C68" s="7"/>
       <c r="D68" s="7"/>
@@ -24213,7 +24219,9 @@
       <c r="BV68" s="18">
         <v>2</v>
       </c>
-      <c r="BW68" s="18"/>
+      <c r="BW68" s="18">
+        <v>1</v>
+      </c>
       <c r="BX68" s="18"/>
       <c r="BY68" s="18"/>
       <c r="BZ68" s="18"/>
@@ -24403,7 +24411,7 @@
       <c r="JB68" s="7"/>
       <c r="JC68" s="20"/>
     </row>
-    <row r="69" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>81</v>
       </c>
@@ -24672,7 +24680,7 @@
       <c r="JB69" s="7"/>
       <c r="JC69" s="20"/>
     </row>
-    <row r="70" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A70" s="8" t="s">
         <v>60</v>
       </c>
@@ -24938,7 +24946,7 @@
       <c r="JB70" s="7"/>
       <c r="JC70" s="20"/>
     </row>
-    <row r="71" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>61</v>
       </c>
@@ -25211,7 +25219,7 @@
       <c r="JB71" s="7"/>
       <c r="JC71" s="20"/>
     </row>
-    <row r="72" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>62</v>
       </c>
@@ -25480,7 +25488,7 @@
       <c r="JB72" s="7"/>
       <c r="JC72" s="20"/>
     </row>
-    <row r="73" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>63</v>
       </c>
@@ -25749,7 +25757,7 @@
       <c r="JB73" s="7"/>
       <c r="JC73" s="20"/>
     </row>
-    <row r="74" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A74" s="8" t="s">
         <v>64</v>
       </c>
@@ -26015,7 +26023,7 @@
       <c r="JB74" s="7"/>
       <c r="JC74" s="20"/>
     </row>
-    <row r="75" spans="1:263" s="12" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:263" s="12" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="6" t="s">
         <v>83</v>
       </c>
@@ -26334,7 +26342,7 @@
       <c r="JB75" s="7"/>
       <c r="JC75" s="20"/>
     </row>
-    <row r="76" spans="1:263" s="12" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:263" s="12" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="6" t="s">
         <v>84</v>
       </c>
@@ -26631,7 +26639,7 @@
       <c r="JB76" s="7"/>
       <c r="JC76" s="20"/>
     </row>
-    <row r="77" spans="1:263" s="12" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:263" s="12" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="6" t="s">
         <v>85</v>
       </c>
@@ -26906,7 +26914,7 @@
       <c r="JB77" s="7"/>
       <c r="JC77" s="20"/>
     </row>
-    <row r="78" spans="1:263" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:263" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>65</v>
       </c>
@@ -27178,7 +27186,7 @@
       <c r="JB78" s="7"/>
       <c r="JC78" s="20"/>
     </row>
-    <row r="79" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>66</v>
       </c>
@@ -27448,7 +27456,7 @@
       <c r="JB79" s="7"/>
       <c r="JC79" s="20"/>
     </row>
-    <row r="80" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>67</v>
       </c>
@@ -27740,7 +27748,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="81" spans="1:263" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:263" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
         <v>68</v>
       </c>
@@ -28020,7 +28028,7 @@
       <c r="JB81" s="7"/>
       <c r="JC81" s="20"/>
     </row>
-    <row r="82" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
         <v>69</v>
       </c>
@@ -28294,7 +28302,7 @@
       <c r="JB82" s="7"/>
       <c r="JC82" s="20"/>
     </row>
-    <row r="83" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A83" s="9" t="s">
         <v>70</v>
       </c>
@@ -28570,7 +28578,7 @@
       <c r="JB83" s="7"/>
       <c r="JC83" s="20"/>
     </row>
-    <row r="84" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:263" x14ac:dyDescent="0.25">
       <c r="A84" s="6" t="s">
         <v>71</v>
       </c>
@@ -28840,7 +28848,7 @@
       <c r="JB84" s="7"/>
       <c r="JC84" s="20"/>
     </row>
-    <row r="85" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:263" x14ac:dyDescent="0.25">
       <c r="B85" s="7"/>
       <c r="E85" s="25"/>
       <c r="F85" s="25"/>
@@ -29028,7 +29036,7 @@
       <c r="GF85" s="25"/>
       <c r="GG85" s="25"/>
     </row>
-    <row r="86" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:263" x14ac:dyDescent="0.25">
       <c r="B86" s="24"/>
       <c r="E86" s="25"/>
       <c r="F86" s="25"/>
@@ -29216,7 +29224,7 @@
       <c r="GF86" s="25"/>
       <c r="GG86" s="25"/>
     </row>
-    <row r="87" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:263" x14ac:dyDescent="0.25">
       <c r="B87" s="7"/>
       <c r="E87" s="25"/>
       <c r="F87" s="25"/>
@@ -29404,7 +29412,7 @@
       <c r="GF87" s="25"/>
       <c r="GG87" s="25"/>
     </row>
-    <row r="88" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:263" x14ac:dyDescent="0.25">
       <c r="B88" s="7"/>
       <c r="E88" s="25"/>
       <c r="F88" s="25"/>
@@ -29592,7 +29600,7 @@
       <c r="GF88" s="25"/>
       <c r="GG88" s="25"/>
     </row>
-    <row r="89" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:263" x14ac:dyDescent="0.25">
       <c r="B89" s="7"/>
       <c r="E89" s="25"/>
       <c r="F89" s="25"/>
@@ -29780,7 +29788,7 @@
       <c r="GF89" s="25"/>
       <c r="GG89" s="25"/>
     </row>
-    <row r="90" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:263" x14ac:dyDescent="0.25">
       <c r="B90" s="7"/>
       <c r="E90" s="25"/>
       <c r="F90" s="25"/>
@@ -29968,7 +29976,7 @@
       <c r="GF90" s="25"/>
       <c r="GG90" s="25"/>
     </row>
-    <row r="91" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:263" x14ac:dyDescent="0.25">
       <c r="B91" s="7"/>
       <c r="E91" s="25"/>
       <c r="F91" s="25"/>
@@ -30156,7 +30164,7 @@
       <c r="GF91" s="25"/>
       <c r="GG91" s="25"/>
     </row>
-    <row r="92" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:263" x14ac:dyDescent="0.25">
       <c r="B92" s="7"/>
       <c r="E92" s="25"/>
       <c r="F92" s="25"/>
@@ -30344,7 +30352,7 @@
       <c r="GF92" s="25"/>
       <c r="GG92" s="25"/>
     </row>
-    <row r="93" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:263" x14ac:dyDescent="0.25">
       <c r="B93" s="7"/>
       <c r="E93" s="25"/>
       <c r="F93" s="25"/>
@@ -30532,7 +30540,7 @@
       <c r="GF93" s="25"/>
       <c r="GG93" s="25"/>
     </row>
-    <row r="94" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:263" x14ac:dyDescent="0.25">
       <c r="B94" s="7"/>
       <c r="E94" s="25"/>
       <c r="F94" s="25"/>
@@ -30720,7 +30728,7 @@
       <c r="GF94" s="25"/>
       <c r="GG94" s="25"/>
     </row>
-    <row r="95" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:263" x14ac:dyDescent="0.25">
       <c r="B95" s="7"/>
       <c r="E95" s="25"/>
       <c r="F95" s="25"/>
@@ -30908,7 +30916,7 @@
       <c r="GF95" s="25"/>
       <c r="GG95" s="25"/>
     </row>
-    <row r="96" spans="1:263" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:263" x14ac:dyDescent="0.25">
       <c r="B96" s="7"/>
       <c r="E96" s="25"/>
       <c r="F96" s="25"/>
@@ -31096,7 +31104,7 @@
       <c r="GF96" s="25"/>
       <c r="GG96" s="25"/>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" s="7"/>
     </row>
   </sheetData>
@@ -31407,15 +31415,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
@@ -31424,6 +31423,15 @@
     <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -31446,14 +31454,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEFE62B7-6772-44D0-ACCE-A546E807D9BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{035973C1-EA40-447A-BB47-72CAA2093BEE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -31468,4 +31468,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEFE62B7-6772-44D0-ACCE-A546E807D9BB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Sync from OneDrive: DSafarik_2026TimeTracking.xlsx [2026-04-14 17:00 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -30817,4 +30817,277 @@
   <pageSetup orientation="portrait"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
+    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
+    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A9E0ACD-E93B-4A52-BE57-CF7CA8B1896C}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53BCD6C9-EB2C-40FD-8E2A-3F362A31BC0C}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13F4132F-0D55-4AE4-B77B-89005D7C3395}"/>
 </file>
</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-04-14 19:18 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -13611,7 +13611,9 @@
       <c r="BW31" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="BX31" s="18" t="n"/>
+      <c r="BX31" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="BY31" s="18" t="n"/>
       <c r="BZ31" s="18" t="n"/>
       <c r="CA31" s="18" t="n"/>
@@ -22761,7 +22763,9 @@
       <c r="BU64" s="18" t="n"/>
       <c r="BV64" s="18" t="n"/>
       <c r="BW64" s="18" t="n"/>
-      <c r="BX64" s="18" t="n"/>
+      <c r="BX64" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="BY64" s="18" t="n"/>
       <c r="BZ64" s="18" t="n"/>
       <c r="CA64" s="18" t="n"/>
@@ -23345,7 +23349,9 @@
       <c r="BW66" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="BX66" s="18" t="n"/>
+      <c r="BX66" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="BY66" s="18" t="n"/>
       <c r="BZ66" s="18" t="n"/>
       <c r="CA66" s="18" t="n"/>
@@ -30817,277 +30823,4 @@
   <pageSetup orientation="portrait"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
-    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A9E0ACD-E93B-4A52-BE57-CF7CA8B1896C}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53BCD6C9-EB2C-40FD-8E2A-3F362A31BC0C}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13F4132F-0D55-4AE4-B77B-89005D7C3395}"/>
 </file>
</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-04-14 19:29 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -9070,7 +9070,9 @@
       <c r="BW15" s="18" t="n">
         <v>0.25</v>
       </c>
-      <c r="BX15" s="18" t="n"/>
+      <c r="BX15" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="BY15" s="18" t="n"/>
       <c r="BZ15" s="18" t="n"/>
       <c r="CA15" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-04-14 19:30 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -7950,7 +7950,9 @@
       <c r="BW11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="BX11" s="18" t="n"/>
+      <c r="BX11" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="BY11" s="18" t="n"/>
       <c r="BZ11" s="18" t="n"/>
       <c r="CA11" s="18" t="n"/>

</xml_diff>

<commit_message>
Sync from OneDrive: DSafarik_2026TimeTracking.xlsx [2026-04-14 21:00 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -30827,4 +30827,277 @@
   <pageSetup orientation="portrait"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
+    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
+    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B13A8BA-B083-4CA0-A602-4A2E9992D6F1}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30A0A177-15BC-4658-8591-0D50220193E4}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD925083-1700-4485-99DA-7DD60819B4C7}"/>
 </file>
</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-04-14 21:59 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8524,7 +8524,9 @@
       <c r="BU13" s="18" t="n"/>
       <c r="BV13" s="18" t="n"/>
       <c r="BW13" s="18" t="n"/>
-      <c r="BX13" s="18" t="n"/>
+      <c r="BX13" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="BY13" s="18" t="n"/>
       <c r="BZ13" s="18" t="n"/>
       <c r="CA13" s="18" t="n"/>
@@ -13616,7 +13618,7 @@
         <v>3</v>
       </c>
       <c r="BX31" s="18" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="BY31" s="18" t="n"/>
       <c r="BZ31" s="18" t="n"/>
@@ -14215,7 +14217,9 @@
       <c r="BW33" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="BX33" s="18" t="n"/>
+      <c r="BX33" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="BY33" s="18" t="n"/>
       <c r="BZ33" s="18" t="n"/>
       <c r="CA33" s="18" t="n"/>
@@ -30827,277 +30831,4 @@
   <pageSetup orientation="portrait"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
-    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B13A8BA-B083-4CA0-A602-4A2E9992D6F1}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{30A0A177-15BC-4658-8591-0D50220193E4}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD925083-1700-4485-99DA-7DD60819B4C7}"/>
 </file>
</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-04-20 20:26 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -9630,7 +9630,9 @@
       <c r="BW17" s="18" t="n"/>
       <c r="BX17" s="18" t="n"/>
       <c r="BY17" s="18" t="n"/>
-      <c r="BZ17" s="18" t="n"/>
+      <c r="BZ17" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CA17" s="18" t="n"/>
       <c r="CB17" s="18" t="n"/>
       <c r="CC17" s="18" t="n"/>
@@ -9906,7 +9908,9 @@
       <c r="BW18" s="18" t="n"/>
       <c r="BX18" s="18" t="n"/>
       <c r="BY18" s="18" t="n"/>
-      <c r="BZ18" s="18" t="n"/>
+      <c r="BZ18" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CA18" s="18" t="n"/>
       <c r="CB18" s="18" t="n"/>
       <c r="CC18" s="18" t="n"/>
@@ -13621,7 +13625,9 @@
         <v>3</v>
       </c>
       <c r="BY31" s="18" t="n"/>
-      <c r="BZ31" s="18" t="n"/>
+      <c r="BZ31" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CA31" s="18" t="n"/>
       <c r="CB31" s="18" t="n"/>
       <c r="CC31" s="18" t="n"/>
@@ -14221,7 +14227,9 @@
         <v>1</v>
       </c>
       <c r="BY33" s="18" t="n"/>
-      <c r="BZ33" s="18" t="n"/>
+      <c r="BZ33" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CA33" s="18" t="n"/>
       <c r="CB33" s="18" t="n"/>
       <c r="CC33" s="18" t="n"/>
@@ -23902,7 +23910,9 @@
       </c>
       <c r="BX68" s="18" t="n"/>
       <c r="BY68" s="18" t="n"/>
-      <c r="BZ68" s="18" t="n"/>
+      <c r="BZ68" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CA68" s="18" t="n"/>
       <c r="CB68" s="18" t="n"/>
       <c r="CC68" s="18" t="n"/>
@@ -26146,7 +26156,9 @@
       <c r="BW76" s="18" t="n"/>
       <c r="BX76" s="18" t="n"/>
       <c r="BY76" s="18" t="n"/>
-      <c r="BZ76" s="18" t="n"/>
+      <c r="BZ76" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CA76" s="18" t="n"/>
       <c r="CB76" s="18" t="n"/>
       <c r="CC76" s="18" t="n"/>
@@ -28099,7 +28111,9 @@
       <c r="BW83" s="18" t="n"/>
       <c r="BX83" s="18" t="n"/>
       <c r="BY83" s="18" t="n"/>
-      <c r="BZ83" s="18" t="n"/>
+      <c r="BZ83" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CA83" s="18" t="n"/>
       <c r="CB83" s="18" t="n"/>
       <c r="CC83" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-04-20 20:28 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -7955,7 +7955,9 @@
       </c>
       <c r="BY11" s="18" t="n"/>
       <c r="BZ11" s="18" t="n"/>
-      <c r="CA11" s="18" t="n"/>
+      <c r="CA11" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CB11" s="18" t="n"/>
       <c r="CC11" s="18" t="n"/>
       <c r="CD11" s="18" t="n"/>
@@ -13628,7 +13630,9 @@
       <c r="BZ31" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CA31" s="18" t="n"/>
+      <c r="CA31" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="CB31" s="18" t="n"/>
       <c r="CC31" s="18" t="n"/>
       <c r="CD31" s="18" t="n"/>
@@ -14230,7 +14234,9 @@
       <c r="BZ33" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CA33" s="18" t="n"/>
+      <c r="CA33" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CB33" s="18" t="n"/>
       <c r="CC33" s="18" t="n"/>
       <c r="CD33" s="18" t="n"/>
@@ -23913,7 +23919,9 @@
       <c r="BZ68" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="CA68" s="18" t="n"/>
+      <c r="CA68" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CB68" s="18" t="n"/>
       <c r="CC68" s="18" t="n"/>
       <c r="CD68" s="18" t="n"/>
@@ -26710,7 +26718,9 @@
       <c r="BX78" s="18" t="n"/>
       <c r="BY78" s="18" t="n"/>
       <c r="BZ78" s="18" t="n"/>
-      <c r="CA78" s="18" t="n"/>
+      <c r="CA78" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CB78" s="18" t="n"/>
       <c r="CC78" s="18" t="n"/>
       <c r="CD78" s="18" t="n"/>

</xml_diff>

<commit_message>
Sync from OneDrive: DSafarik_2026TimeTracking.xlsx [2026-04-21 03:00 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -30855,4 +30855,277 @@
   <pageSetup orientation="portrait"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
+    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
+    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2ED7FF37-3A67-4D37-AF31-CBE2951D9F72}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{751BC6D9-0B57-4E7D-BE5A-A1D58B721B88}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{110DA2EF-CA1E-4B07-A715-474BBBCC884D}"/>
 </file>
</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-04-22 19:59 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -7959,7 +7959,9 @@
         <v>1</v>
       </c>
       <c r="CB11" s="18" t="n"/>
-      <c r="CC11" s="18" t="n"/>
+      <c r="CC11" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CD11" s="18" t="n"/>
       <c r="CE11" s="18" t="n"/>
       <c r="CF11" s="18" t="n"/>
@@ -9083,7 +9085,9 @@
       <c r="BZ15" s="18" t="n"/>
       <c r="CA15" s="18" t="n"/>
       <c r="CB15" s="18" t="n"/>
-      <c r="CC15" s="18" t="n"/>
+      <c r="CC15" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CD15" s="18" t="n"/>
       <c r="CE15" s="18" t="n"/>
       <c r="CF15" s="18" t="n"/>
@@ -10198,7 +10202,9 @@
       <c r="BZ19" s="18" t="n"/>
       <c r="CA19" s="18" t="n"/>
       <c r="CB19" s="18" t="n"/>
-      <c r="CC19" s="18" t="n"/>
+      <c r="CC19" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CD19" s="18" t="n"/>
       <c r="CE19" s="18" t="n"/>
       <c r="CF19" s="18" t="n"/>
@@ -13634,7 +13640,9 @@
         <v>3</v>
       </c>
       <c r="CB31" s="18" t="n"/>
-      <c r="CC31" s="18" t="n"/>
+      <c r="CC31" s="18" t="n">
+        <v>4.5</v>
+      </c>
       <c r="CD31" s="18" t="n"/>
       <c r="CE31" s="18" t="n"/>
       <c r="CF31" s="18" t="n"/>
@@ -23378,7 +23386,9 @@
       <c r="BZ66" s="18" t="n"/>
       <c r="CA66" s="18" t="n"/>
       <c r="CB66" s="18" t="n"/>
-      <c r="CC66" s="18" t="n"/>
+      <c r="CC66" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CD66" s="18" t="n"/>
       <c r="CE66" s="18" t="n"/>
       <c r="CF66" s="18" t="n"/>
@@ -30855,277 +30865,4 @@
   <pageSetup orientation="portrait"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
-    <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
-    <xsd:import namespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="be2d32d5-45e4-45f8-8cca-e731efdae529" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="10" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="11" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="7ff297e6-98dc-4a77-8782-4199b303df17" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{433bb87c-b111-4230-a796-99831eb60517}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2ED7FF37-3A67-4D37-AF31-CBE2951D9F72}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{751BC6D9-0B57-4E7D-BE5A-A1D58B721B88}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{110DA2EF-CA1E-4B07-A715-474BBBCC884D}"/>
 </file>
</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-04-24 22:06 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8241,7 +8241,9 @@
       <c r="CB12" s="18" t="n"/>
       <c r="CC12" s="18" t="n"/>
       <c r="CD12" s="18" t="n"/>
-      <c r="CE12" s="18" t="n"/>
+      <c r="CE12" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CF12" s="18" t="n"/>
       <c r="CG12" s="18" t="n"/>
       <c r="CH12" s="18" t="n"/>
@@ -13644,7 +13646,9 @@
         <v>4.5</v>
       </c>
       <c r="CD31" s="18" t="n"/>
-      <c r="CE31" s="18" t="n"/>
+      <c r="CE31" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="CF31" s="18" t="n"/>
       <c r="CG31" s="18" t="n"/>
       <c r="CH31" s="18" t="n"/>
@@ -14248,7 +14252,9 @@
       <c r="CB33" s="18" t="n"/>
       <c r="CC33" s="18" t="n"/>
       <c r="CD33" s="18" t="n"/>
-      <c r="CE33" s="18" t="n"/>
+      <c r="CE33" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CF33" s="18" t="n"/>
       <c r="CG33" s="18" t="n"/>
       <c r="CH33" s="18" t="n"/>
@@ -23390,7 +23396,9 @@
         <v>1</v>
       </c>
       <c r="CD66" s="18" t="n"/>
-      <c r="CE66" s="18" t="n"/>
+      <c r="CE66" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CF66" s="18" t="n"/>
       <c r="CG66" s="18" t="n"/>
       <c r="CH66" s="18" t="n"/>
@@ -23663,7 +23671,9 @@
       <c r="CB67" s="18" t="n"/>
       <c r="CC67" s="18" t="n"/>
       <c r="CD67" s="18" t="n"/>
-      <c r="CE67" s="18" t="n"/>
+      <c r="CE67" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CF67" s="18" t="n"/>
       <c r="CG67" s="18" t="n"/>
       <c r="CH67" s="18" t="n"/>
@@ -26181,7 +26191,9 @@
       <c r="CB76" s="18" t="n"/>
       <c r="CC76" s="18" t="n"/>
       <c r="CD76" s="18" t="n"/>
-      <c r="CE76" s="18" t="n"/>
+      <c r="CE76" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CF76" s="18" t="n"/>
       <c r="CG76" s="18" t="n"/>
       <c r="CH76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-04-24 22:09 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8244,7 +8244,9 @@
       <c r="CE12" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="CF12" s="18" t="n"/>
+      <c r="CF12" s="18" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CG12" s="18" t="n"/>
       <c r="CH12" s="18" t="n"/>
       <c r="CI12" s="18" t="n"/>
@@ -10801,7 +10803,9 @@
       <c r="CC21" s="18" t="n"/>
       <c r="CD21" s="18" t="n"/>
       <c r="CE21" s="18" t="n"/>
-      <c r="CF21" s="18" t="n"/>
+      <c r="CF21" s="18" t="n">
+        <v>2.75</v>
+      </c>
       <c r="CG21" s="18" t="n"/>
       <c r="CH21" s="18" t="n"/>
       <c r="CI21" s="18" t="n"/>
@@ -14255,7 +14259,9 @@
       <c r="CE33" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="CF33" s="18" t="n"/>
+      <c r="CF33" s="18" t="n">
+        <v>2.25</v>
+      </c>
       <c r="CG33" s="18" t="n"/>
       <c r="CH33" s="18" t="n"/>
       <c r="CI33" s="18" t="n"/>
@@ -23399,7 +23405,9 @@
       <c r="CE66" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CF66" s="18" t="n"/>
+      <c r="CF66" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CG66" s="18" t="n"/>
       <c r="CH66" s="18" t="n"/>
       <c r="CI66" s="18" t="n"/>
@@ -23674,7 +23682,9 @@
       <c r="CE67" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="CF67" s="18" t="n"/>
+      <c r="CF67" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CG67" s="18" t="n"/>
       <c r="CH67" s="18" t="n"/>
       <c r="CI67" s="18" t="n"/>
@@ -26194,7 +26204,9 @@
       <c r="CE76" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="CF76" s="18" t="n"/>
+      <c r="CF76" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CG76" s="18" t="n"/>
       <c r="CH76" s="18" t="n"/>
       <c r="CI76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-04-27 22:04 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -7965,7 +7965,9 @@
       <c r="CD11" s="18" t="n"/>
       <c r="CE11" s="18" t="n"/>
       <c r="CF11" s="18" t="n"/>
-      <c r="CG11" s="18" t="n"/>
+      <c r="CG11" s="18" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CH11" s="18" t="n"/>
       <c r="CI11" s="18" t="n"/>
       <c r="CJ11" s="19" t="n"/>
@@ -8247,7 +8249,9 @@
       <c r="CF12" s="18" t="n">
         <v>0.25</v>
       </c>
-      <c r="CG12" s="18" t="n"/>
+      <c r="CG12" s="18" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CH12" s="18" t="n"/>
       <c r="CI12" s="18" t="n"/>
       <c r="CJ12" s="19" t="n"/>
@@ -13654,7 +13658,9 @@
         <v>3</v>
       </c>
       <c r="CF31" s="18" t="n"/>
-      <c r="CG31" s="18" t="n"/>
+      <c r="CG31" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CH31" s="18" t="n"/>
       <c r="CI31" s="18" t="n"/>
       <c r="CJ31" s="19" t="n"/>
@@ -14262,7 +14268,9 @@
       <c r="CF33" s="18" t="n">
         <v>2.25</v>
       </c>
-      <c r="CG33" s="18" t="n"/>
+      <c r="CG33" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CH33" s="18" t="n"/>
       <c r="CI33" s="18" t="n"/>
       <c r="CJ33" s="19" t="n"/>
@@ -25902,7 +25910,9 @@
       <c r="CD75" s="18" t="n"/>
       <c r="CE75" s="18" t="n"/>
       <c r="CF75" s="18" t="n"/>
-      <c r="CG75" s="18" t="n"/>
+      <c r="CG75" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CH75" s="18" t="n"/>
       <c r="CI75" s="18" t="n"/>
       <c r="CJ75" s="19" t="n"/>
@@ -28164,7 +28174,9 @@
       <c r="CD83" s="18" t="n"/>
       <c r="CE83" s="18" t="n"/>
       <c r="CF83" s="18" t="n"/>
-      <c r="CG83" s="18" t="n"/>
+      <c r="CG83" s="18" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CH83" s="18" t="n"/>
       <c r="CI83" s="18" t="n"/>
       <c r="CJ83" s="19" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-04-28 14:40 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -10811,7 +10811,9 @@
         <v>2.75</v>
       </c>
       <c r="CG21" s="18" t="n"/>
-      <c r="CH21" s="18" t="n"/>
+      <c r="CH21" s="18" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CI21" s="18" t="n"/>
       <c r="CJ21" s="19" t="n"/>
       <c r="CK21" s="18" t="n"/>
@@ -14271,7 +14273,9 @@
       <c r="CG33" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CH33" s="18" t="n"/>
+      <c r="CH33" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CI33" s="18" t="n"/>
       <c r="CJ33" s="19" t="n"/>
       <c r="CK33" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-04-29 23:15 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -7969,7 +7969,9 @@
         <v>1.25</v>
       </c>
       <c r="CH11" s="18" t="n"/>
-      <c r="CI11" s="18" t="n"/>
+      <c r="CI11" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CJ11" s="19" t="n"/>
       <c r="CK11" s="18" t="n"/>
       <c r="CL11" s="18" t="n"/>
@@ -8253,7 +8255,9 @@
         <v>0.25</v>
       </c>
       <c r="CH12" s="18" t="n"/>
-      <c r="CI12" s="18" t="n"/>
+      <c r="CI12" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CJ12" s="19" t="n"/>
       <c r="CK12" s="18" t="n"/>
       <c r="CL12" s="18" t="n"/>
@@ -10814,7 +10818,9 @@
       <c r="CH21" s="18" t="n">
         <v>0.25</v>
       </c>
-      <c r="CI21" s="18" t="n"/>
+      <c r="CI21" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CJ21" s="19" t="n"/>
       <c r="CK21" s="18" t="n"/>
       <c r="CL21" s="18" t="n"/>
@@ -14276,7 +14282,9 @@
       <c r="CH33" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="CI33" s="18" t="n"/>
+      <c r="CI33" s="18" t="n">
+        <v>5</v>
+      </c>
       <c r="CJ33" s="19" t="n"/>
       <c r="CK33" s="18" t="n"/>
       <c r="CL33" s="18" t="n"/>
@@ -22830,7 +22838,9 @@
       <c r="CF64" s="18" t="n"/>
       <c r="CG64" s="18" t="n"/>
       <c r="CH64" s="18" t="n"/>
-      <c r="CI64" s="18" t="n"/>
+      <c r="CI64" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CJ64" s="19" t="n"/>
       <c r="CK64" s="18" t="n"/>
       <c r="CL64" s="18" t="n"/>
@@ -26223,7 +26233,9 @@
       </c>
       <c r="CG76" s="18" t="n"/>
       <c r="CH76" s="18" t="n"/>
-      <c r="CI76" s="18" t="n"/>
+      <c r="CI76" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CJ76" s="19" t="n"/>
       <c r="CK76" s="18" t="n"/>
       <c r="CL76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-04-30 13:28 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -14285,7 +14285,9 @@
       <c r="CI33" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="CJ33" s="19" t="n"/>
+      <c r="CJ33" s="19" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CK33" s="18" t="n"/>
       <c r="CL33" s="18" t="n"/>
       <c r="CM33" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-04-30 17:29 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -7972,7 +7972,9 @@
       <c r="CI11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="CJ11" s="19" t="n"/>
+      <c r="CJ11" s="19" t="n">
+        <v>1</v>
+      </c>
       <c r="CK11" s="18" t="n"/>
       <c r="CL11" s="18" t="n"/>
       <c r="CM11" s="18" t="n"/>
@@ -9106,7 +9108,9 @@
       <c r="CG15" s="18" t="n"/>
       <c r="CH15" s="18" t="n"/>
       <c r="CI15" s="18" t="n"/>
-      <c r="CJ15" s="19" t="n"/>
+      <c r="CJ15" s="19" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CK15" s="18" t="n"/>
       <c r="CL15" s="18" t="n"/>
       <c r="CM15" s="18" t="n"/>
@@ -13671,7 +13675,9 @@
       </c>
       <c r="CH31" s="18" t="n"/>
       <c r="CI31" s="18" t="n"/>
-      <c r="CJ31" s="19" t="n"/>
+      <c r="CJ31" s="19" t="n">
+        <v>1</v>
+      </c>
       <c r="CK31" s="18" t="n"/>
       <c r="CL31" s="18" t="n"/>
       <c r="CM31" s="18" t="n"/>
@@ -14286,7 +14292,7 @@
         <v>5</v>
       </c>
       <c r="CJ33" s="19" t="n">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="CK33" s="18" t="n"/>
       <c r="CL33" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-01 16:03 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -9111,7 +9111,9 @@
       <c r="CJ15" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="CK15" s="18" t="n"/>
+      <c r="CK15" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CL15" s="18" t="n"/>
       <c r="CM15" s="18" t="n"/>
       <c r="CN15" s="18" t="n"/>
@@ -25938,7 +25940,9 @@
       <c r="CH75" s="18" t="n"/>
       <c r="CI75" s="18" t="n"/>
       <c r="CJ75" s="19" t="n"/>
-      <c r="CK75" s="18" t="n"/>
+      <c r="CK75" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CL75" s="18" t="n"/>
       <c r="CM75" s="18" t="n"/>
       <c r="CN75" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-01 17:18 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -18655,7 +18655,9 @@
       <c r="CH49" s="18" t="n"/>
       <c r="CI49" s="18" t="n"/>
       <c r="CJ49" s="19" t="n"/>
-      <c r="CK49" s="18" t="n"/>
+      <c r="CK49" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="CL49" s="18" t="n"/>
       <c r="CM49" s="18" t="n"/>
       <c r="CN49" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-01 20:20 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -12768,7 +12768,9 @@
       <c r="CH28" s="18" t="n"/>
       <c r="CI28" s="18" t="n"/>
       <c r="CJ28" s="19" t="n"/>
-      <c r="CK28" s="18" t="n"/>
+      <c r="CK28" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CL28" s="18" t="n"/>
       <c r="CM28" s="18" t="n"/>
       <c r="CN28" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-01 20:21 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -13682,7 +13682,9 @@
       <c r="CJ31" s="19" t="n">
         <v>2.75</v>
       </c>
-      <c r="CK31" s="18" t="n"/>
+      <c r="CK31" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CL31" s="18" t="n"/>
       <c r="CM31" s="18" t="n"/>
       <c r="CN31" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-01 21:51 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -27657,7 +27657,9 @@
       <c r="CI81" s="18" t="n"/>
       <c r="CJ81" s="19" t="n"/>
       <c r="CK81" s="18" t="n"/>
-      <c r="CL81" s="18" t="n"/>
+      <c r="CL81" s="18" t="n">
+        <v>8</v>
+      </c>
       <c r="CM81" s="18" t="n"/>
       <c r="CN81" s="18" t="n"/>
       <c r="CO81" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-01 21:52 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -9391,7 +9391,9 @@
       <c r="CJ16" s="19" t="n"/>
       <c r="CK16" s="18" t="n"/>
       <c r="CL16" s="18" t="n"/>
-      <c r="CM16" s="18" t="n"/>
+      <c r="CM16" s="18" t="n">
+        <v>8</v>
+      </c>
       <c r="CN16" s="18" t="n"/>
       <c r="CO16" s="18" t="n"/>
       <c r="CP16" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-01 21:53 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -24004,7 +24004,9 @@
       <c r="CK68" s="18" t="n"/>
       <c r="CL68" s="18" t="n"/>
       <c r="CM68" s="18" t="n"/>
-      <c r="CN68" s="18" t="n"/>
+      <c r="CN68" s="18" t="n">
+        <v>8</v>
+      </c>
       <c r="CO68" s="18" t="n"/>
       <c r="CP68" s="18" t="n"/>
       <c r="CQ68" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-01 21:55 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -27666,7 +27666,9 @@
       </c>
       <c r="CM81" s="18" t="n"/>
       <c r="CN81" s="18" t="n"/>
-      <c r="CO81" s="18" t="n"/>
+      <c r="CO81" s="18" t="n">
+        <v>8</v>
+      </c>
       <c r="CP81" s="18" t="n"/>
       <c r="CQ81" s="18" t="n"/>
       <c r="CR81" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-01 21:56 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -27669,7 +27669,9 @@
       <c r="CO81" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="CP81" s="18" t="n"/>
+      <c r="CP81" s="18" t="n">
+        <v>8</v>
+      </c>
       <c r="CQ81" s="18" t="n"/>
       <c r="CR81" s="18" t="n"/>
       <c r="CS81" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-11 16:33 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -9119,7 +9119,9 @@
       <c r="CN15" s="18" t="n"/>
       <c r="CO15" s="18" t="n"/>
       <c r="CP15" s="18" t="n"/>
-      <c r="CQ15" s="18" t="n"/>
+      <c r="CQ15" s="18" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CR15" s="18" t="n"/>
       <c r="CS15" s="18" t="n"/>
       <c r="CT15" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-11 20:21 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -7981,7 +7981,9 @@
       <c r="CN11" s="18" t="n"/>
       <c r="CO11" s="18" t="n"/>
       <c r="CP11" s="18" t="n"/>
-      <c r="CQ11" s="18" t="n"/>
+      <c r="CQ11" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CR11" s="18" t="n"/>
       <c r="CS11" s="18" t="n"/>
       <c r="CT11" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-12 13:17 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -7982,7 +7982,7 @@
       <c r="CO11" s="18" t="n"/>
       <c r="CP11" s="18" t="n"/>
       <c r="CQ11" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CR11" s="18" t="n"/>
       <c r="CS11" s="18" t="n"/>
@@ -17577,7 +17577,9 @@
       <c r="CN45" s="18" t="n"/>
       <c r="CO45" s="18" t="n"/>
       <c r="CP45" s="18" t="n"/>
-      <c r="CQ45" s="18" t="n"/>
+      <c r="CQ45" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CR45" s="18" t="n"/>
       <c r="CS45" s="18" t="n"/>
       <c r="CT45" s="18" t="n"/>
@@ -22220,7 +22222,9 @@
       <c r="CN62" s="18" t="n"/>
       <c r="CO62" s="18" t="n"/>
       <c r="CP62" s="18" t="n"/>
-      <c r="CQ62" s="18" t="n"/>
+      <c r="CQ62" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CR62" s="18" t="n"/>
       <c r="CS62" s="18" t="n"/>
       <c r="CT62" s="18" t="n"/>
@@ -25962,7 +25966,9 @@
       <c r="CN75" s="18" t="n"/>
       <c r="CO75" s="18" t="n"/>
       <c r="CP75" s="18" t="n"/>
-      <c r="CQ75" s="18" t="n"/>
+      <c r="CQ75" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CR75" s="18" t="n"/>
       <c r="CS75" s="18" t="n"/>
       <c r="CT75" s="18" t="n"/>
@@ -26269,7 +26275,9 @@
       <c r="CN76" s="18" t="n"/>
       <c r="CO76" s="18" t="n"/>
       <c r="CP76" s="18" t="n"/>
-      <c r="CQ76" s="18" t="n"/>
+      <c r="CQ76" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CR76" s="18" t="n"/>
       <c r="CS76" s="18" t="n"/>
       <c r="CT76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-12 16:15 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -7984,7 +7984,9 @@
       <c r="CQ11" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="CR11" s="18" t="n"/>
+      <c r="CR11" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CS11" s="18" t="n"/>
       <c r="CT11" s="18" t="n"/>
       <c r="CU11" s="18" t="n"/>
@@ -13697,7 +13699,9 @@
       <c r="CO31" s="18" t="n"/>
       <c r="CP31" s="18" t="n"/>
       <c r="CQ31" s="18" t="n"/>
-      <c r="CR31" s="18" t="n"/>
+      <c r="CR31" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CS31" s="18" t="n"/>
       <c r="CT31" s="18" t="n"/>
       <c r="CU31" s="18" t="n"/>
@@ -23469,7 +23473,9 @@
       <c r="CO66" s="18" t="n"/>
       <c r="CP66" s="18" t="n"/>
       <c r="CQ66" s="18" t="n"/>
-      <c r="CR66" s="18" t="n"/>
+      <c r="CR66" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CS66" s="18" t="n"/>
       <c r="CT66" s="18" t="n"/>
       <c r="CU66" s="18" t="n"/>
@@ -25971,7 +25977,9 @@
       <c r="CQ75" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="CR75" s="18" t="n"/>
+      <c r="CR75" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CS75" s="18" t="n"/>
       <c r="CT75" s="18" t="n"/>
       <c r="CU75" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-13 14:15 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -13700,7 +13700,7 @@
       <c r="CP31" s="18" t="n"/>
       <c r="CQ31" s="18" t="n"/>
       <c r="CR31" s="18" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="CS31" s="18" t="n"/>
       <c r="CT31" s="18" t="n"/>
@@ -14317,7 +14317,9 @@
       <c r="CO33" s="18" t="n"/>
       <c r="CP33" s="18" t="n"/>
       <c r="CQ33" s="18" t="n"/>
-      <c r="CR33" s="18" t="n"/>
+      <c r="CR33" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CS33" s="18" t="n"/>
       <c r="CT33" s="18" t="n"/>
       <c r="CU33" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-13 14:16 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -14318,7 +14318,7 @@
       <c r="CP33" s="18" t="n"/>
       <c r="CQ33" s="18" t="n"/>
       <c r="CR33" s="18" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="CS33" s="18" t="n"/>
       <c r="CT33" s="18" t="n"/>
@@ -17586,7 +17586,9 @@
       <c r="CQ45" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CR45" s="18" t="n"/>
+      <c r="CR45" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CS45" s="18" t="n"/>
       <c r="CT45" s="18" t="n"/>
       <c r="CU45" s="18" t="n"/>
@@ -22233,7 +22235,9 @@
       <c r="CQ62" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="CR62" s="18" t="n"/>
+      <c r="CR62" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CS62" s="18" t="n"/>
       <c r="CT62" s="18" t="n"/>
       <c r="CU62" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-13 21:51 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -7987,7 +7987,9 @@
       <c r="CR11" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="CS11" s="18" t="n"/>
+      <c r="CS11" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CT11" s="18" t="n"/>
       <c r="CU11" s="18" t="n"/>
       <c r="CV11" s="18" t="n"/>
@@ -13702,7 +13704,9 @@
       <c r="CR31" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CS31" s="18" t="n"/>
+      <c r="CS31" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="CT31" s="18" t="n"/>
       <c r="CU31" s="18" t="n"/>
       <c r="CV31" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-13 22:58 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8275,7 +8275,9 @@
       <c r="CP12" s="18" t="n"/>
       <c r="CQ12" s="18" t="n"/>
       <c r="CR12" s="18" t="n"/>
-      <c r="CS12" s="18" t="n"/>
+      <c r="CS12" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CT12" s="18" t="n"/>
       <c r="CU12" s="18" t="n"/>
       <c r="CV12" s="18" t="n"/>
@@ -10846,7 +10848,9 @@
       <c r="CP21" s="18" t="n"/>
       <c r="CQ21" s="18" t="n"/>
       <c r="CR21" s="18" t="n"/>
-      <c r="CS21" s="18" t="n"/>
+      <c r="CS21" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CT21" s="18" t="n"/>
       <c r="CU21" s="18" t="n"/>
       <c r="CV21" s="18" t="n"/>
@@ -14324,7 +14328,9 @@
       <c r="CR33" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CS33" s="18" t="n"/>
+      <c r="CS33" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CT33" s="18" t="n"/>
       <c r="CU33" s="18" t="n"/>
       <c r="CV33" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-15 15:25 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -26306,7 +26306,9 @@
       </c>
       <c r="CR76" s="18" t="n"/>
       <c r="CS76" s="18" t="n"/>
-      <c r="CT76" s="18" t="n"/>
+      <c r="CT76" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CU76" s="18" t="n"/>
       <c r="CV76" s="18" t="n"/>
       <c r="CW76" s="18" t="n"/>
@@ -26583,7 +26585,9 @@
       <c r="CQ77" s="18" t="n"/>
       <c r="CR77" s="18" t="n"/>
       <c r="CS77" s="18" t="n"/>
-      <c r="CT77" s="18" t="n"/>
+      <c r="CT77" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CU77" s="18" t="n"/>
       <c r="CV77" s="18" t="n"/>
       <c r="CW77" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-15 15:27 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -13711,7 +13711,9 @@
       <c r="CS31" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="CT31" s="18" t="n"/>
+      <c r="CT31" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CU31" s="18" t="n"/>
       <c r="CV31" s="18" t="n"/>
       <c r="CW31" s="18" t="n"/>
@@ -14331,7 +14333,9 @@
       <c r="CS33" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CT33" s="18" t="n"/>
+      <c r="CT33" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CU33" s="18" t="n"/>
       <c r="CV33" s="18" t="n"/>
       <c r="CW33" s="18" t="n"/>
@@ -17324,7 +17328,9 @@
       <c r="CQ44" s="18" t="n"/>
       <c r="CR44" s="18" t="n"/>
       <c r="CS44" s="18" t="n"/>
-      <c r="CT44" s="18" t="n"/>
+      <c r="CT44" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CU44" s="18" t="n"/>
       <c r="CV44" s="18" t="n"/>
       <c r="CW44" s="18" t="n"/>
@@ -17600,7 +17606,9 @@
         <v>1</v>
       </c>
       <c r="CS45" s="18" t="n"/>
-      <c r="CT45" s="18" t="n"/>
+      <c r="CT45" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CU45" s="18" t="n"/>
       <c r="CV45" s="18" t="n"/>
       <c r="CW45" s="18" t="n"/>
@@ -18698,7 +18706,9 @@
         <v>0.5</v>
       </c>
       <c r="CS49" s="18" t="n"/>
-      <c r="CT49" s="18" t="n"/>
+      <c r="CT49" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CU49" s="18" t="n"/>
       <c r="CV49" s="18" t="n"/>
       <c r="CW49" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-15 16:52 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8575,7 +8575,9 @@
       <c r="CR13" s="18" t="n"/>
       <c r="CS13" s="18" t="n"/>
       <c r="CT13" s="18" t="n"/>
-      <c r="CU13" s="18" t="n"/>
+      <c r="CU13" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CV13" s="18" t="n"/>
       <c r="CW13" s="18" t="n"/>
       <c r="CX13" s="18" t="n"/>
@@ -13714,7 +13716,9 @@
       <c r="CT31" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CU31" s="18" t="n"/>
+      <c r="CU31" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CV31" s="18" t="n"/>
       <c r="CW31" s="18" t="n"/>
       <c r="CX31" s="18" t="n"/>
@@ -14336,7 +14340,9 @@
       <c r="CT33" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="CU33" s="18" t="n"/>
+      <c r="CU33" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CV33" s="18" t="n"/>
       <c r="CW33" s="18" t="n"/>
       <c r="CX33" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-15 19:37 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -26325,7 +26325,9 @@
       <c r="CT76" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="CU76" s="18" t="n"/>
+      <c r="CU76" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CV76" s="18" t="n"/>
       <c r="CW76" s="18" t="n"/>
       <c r="CX76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-15 19:39 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8279,7 +8279,9 @@
         <v>1</v>
       </c>
       <c r="CT12" s="18" t="n"/>
-      <c r="CU12" s="18" t="n"/>
+      <c r="CU12" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CV12" s="18" t="n"/>
       <c r="CW12" s="18" t="n"/>
       <c r="CX12" s="18" t="n"/>
@@ -17615,7 +17617,9 @@
       <c r="CT45" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="CU45" s="18" t="n"/>
+      <c r="CU45" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CV45" s="18" t="n"/>
       <c r="CW45" s="18" t="n"/>
       <c r="CX45" s="18" t="n"/>
@@ -23510,7 +23514,9 @@
       </c>
       <c r="CS66" s="18" t="n"/>
       <c r="CT66" s="18" t="n"/>
-      <c r="CU66" s="18" t="n"/>
+      <c r="CU66" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CV66" s="18" t="n"/>
       <c r="CW66" s="18" t="n"/>
       <c r="CX66" s="18" t="n"/>
@@ -26326,7 +26332,7 @@
         <v>0.5</v>
       </c>
       <c r="CU76" s="18" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="CV76" s="18" t="n"/>
       <c r="CW76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-18 21:20 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -13719,7 +13719,7 @@
         <v>2</v>
       </c>
       <c r="CU31" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CV31" s="18" t="n"/>
       <c r="CW31" s="18" t="n"/>
@@ -14343,7 +14343,7 @@
         <v>3</v>
       </c>
       <c r="CU33" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="CV33" s="18" t="n"/>
       <c r="CW33" s="18" t="n"/>
@@ -26020,7 +26020,9 @@
       </c>
       <c r="CS75" s="18" t="n"/>
       <c r="CT75" s="18" t="n"/>
-      <c r="CU75" s="18" t="n"/>
+      <c r="CU75" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CV75" s="18" t="n"/>
       <c r="CW75" s="18" t="n"/>
       <c r="CX75" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-18 21:21 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8282,7 +8282,9 @@
       <c r="CU12" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="CV12" s="18" t="n"/>
+      <c r="CV12" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CW12" s="18" t="n"/>
       <c r="CX12" s="18" t="n"/>
       <c r="CY12" s="18" t="n"/>
@@ -8854,7 +8856,9 @@
       <c r="CS14" s="18" t="n"/>
       <c r="CT14" s="18" t="n"/>
       <c r="CU14" s="18" t="n"/>
-      <c r="CV14" s="18" t="n"/>
+      <c r="CV14" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CW14" s="18" t="n"/>
       <c r="CX14" s="18" t="n"/>
       <c r="CY14" s="18" t="n"/>
@@ -13721,7 +13725,9 @@
       <c r="CU31" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CV31" s="18" t="n"/>
+      <c r="CV31" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CW31" s="18" t="n"/>
       <c r="CX31" s="18" t="n"/>
       <c r="CY31" s="18" t="n"/>
@@ -24068,7 +24074,9 @@
       <c r="CS68" s="18" t="n"/>
       <c r="CT68" s="18" t="n"/>
       <c r="CU68" s="18" t="n"/>
-      <c r="CV68" s="18" t="n"/>
+      <c r="CV68" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CW68" s="18" t="n"/>
       <c r="CX68" s="18" t="n"/>
       <c r="CY68" s="18" t="n"/>
@@ -26023,7 +26031,9 @@
       <c r="CU75" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="CV75" s="18" t="n"/>
+      <c r="CV75" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CW75" s="18" t="n"/>
       <c r="CX75" s="18" t="n"/>
       <c r="CY75" s="18" t="n"/>
@@ -26336,7 +26346,9 @@
       <c r="CU76" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="CV76" s="18" t="n"/>
+      <c r="CV76" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CW76" s="18" t="n"/>
       <c r="CX76" s="18" t="n"/>
       <c r="CY76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-18 21:22 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -15441,7 +15441,9 @@
       <c r="CS37" s="18" t="n"/>
       <c r="CT37" s="18" t="n"/>
       <c r="CU37" s="18" t="n"/>
-      <c r="CV37" s="18" t="n"/>
+      <c r="CV37" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CW37" s="18" t="n"/>
       <c r="CX37" s="18" t="n"/>
       <c r="CY37" s="18" t="n"/>
@@ -24075,7 +24077,7 @@
       <c r="CT68" s="18" t="n"/>
       <c r="CU68" s="18" t="n"/>
       <c r="CV68" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="CW68" s="18" t="n"/>
       <c r="CX68" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-19 23:04 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -7993,7 +7993,9 @@
       <c r="CT11" s="18" t="n"/>
       <c r="CU11" s="18" t="n"/>
       <c r="CV11" s="18" t="n"/>
-      <c r="CW11" s="18" t="n"/>
+      <c r="CW11" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CX11" s="18" t="n"/>
       <c r="CY11" s="18" t="n"/>
       <c r="CZ11" s="18" t="n"/>
@@ -8583,7 +8585,9 @@
         <v>1</v>
       </c>
       <c r="CV13" s="18" t="n"/>
-      <c r="CW13" s="18" t="n"/>
+      <c r="CW13" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CX13" s="18" t="n"/>
       <c r="CY13" s="18" t="n"/>
       <c r="CZ13" s="18" t="n"/>
@@ -10862,7 +10866,9 @@
       <c r="CT21" s="18" t="n"/>
       <c r="CU21" s="18" t="n"/>
       <c r="CV21" s="18" t="n"/>
-      <c r="CW21" s="18" t="n"/>
+      <c r="CW21" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CX21" s="18" t="n"/>
       <c r="CY21" s="18" t="n"/>
       <c r="CZ21" s="18" t="n"/>
@@ -13728,7 +13734,9 @@
       <c r="CV31" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CW31" s="18" t="n"/>
+      <c r="CW31" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CX31" s="18" t="n"/>
       <c r="CY31" s="18" t="n"/>
       <c r="CZ31" s="18" t="n"/>
@@ -14352,7 +14360,9 @@
         <v>2</v>
       </c>
       <c r="CV33" s="18" t="n"/>
-      <c r="CW33" s="18" t="n"/>
+      <c r="CW33" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CX33" s="18" t="n"/>
       <c r="CY33" s="18" t="n"/>
       <c r="CZ33" s="18" t="n"/>
@@ -17629,7 +17639,9 @@
         <v>0.5</v>
       </c>
       <c r="CV45" s="18" t="n"/>
-      <c r="CW45" s="18" t="n"/>
+      <c r="CW45" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CX45" s="18" t="n"/>
       <c r="CY45" s="18" t="n"/>
       <c r="CZ45" s="18" t="n"/>
@@ -23526,7 +23538,9 @@
         <v>0.5</v>
       </c>
       <c r="CV66" s="18" t="n"/>
-      <c r="CW66" s="18" t="n"/>
+      <c r="CW66" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CX66" s="18" t="n"/>
       <c r="CY66" s="18" t="n"/>
       <c r="CZ66" s="18" t="n"/>
@@ -26351,7 +26365,9 @@
       <c r="CV76" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="CW76" s="18" t="n"/>
+      <c r="CW76" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CX76" s="18" t="n"/>
       <c r="CY76" s="18" t="n"/>
       <c r="CZ76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-26 22:43 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -7996,7 +7996,9 @@
       <c r="CW11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="CX11" s="18" t="n"/>
+      <c r="CX11" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CY11" s="18" t="n"/>
       <c r="CZ11" s="18" t="n"/>
       <c r="DA11" s="18" t="n"/>
@@ -8864,7 +8866,9 @@
         <v>0.5</v>
       </c>
       <c r="CW14" s="18" t="n"/>
-      <c r="CX14" s="18" t="n"/>
+      <c r="CX14" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CY14" s="18" t="n"/>
       <c r="CZ14" s="18" t="n"/>
       <c r="DA14" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-26 22:48 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -13741,7 +13741,9 @@
       <c r="CW31" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CX31" s="18" t="n"/>
+      <c r="CX31" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CY31" s="18" t="n"/>
       <c r="CZ31" s="18" t="n"/>
       <c r="DA31" s="18" t="n"/>
@@ -17646,7 +17648,9 @@
       <c r="CW45" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CX45" s="18" t="n"/>
+      <c r="CX45" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CY45" s="18" t="n"/>
       <c r="CZ45" s="18" t="n"/>
       <c r="DA45" s="18" t="n"/>
@@ -23545,7 +23549,9 @@
       <c r="CW66" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CX66" s="18" t="n"/>
+      <c r="CX66" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CY66" s="18" t="n"/>
       <c r="CZ66" s="18" t="n"/>
       <c r="DA66" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-26 22:49 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8869,7 +8869,9 @@
       <c r="CX14" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="CY14" s="18" t="n"/>
+      <c r="CY14" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CZ14" s="18" t="n"/>
       <c r="DA14" s="18" t="n"/>
       <c r="DB14" s="18" t="n"/>
@@ -11457,7 +11459,9 @@
       <c r="CV23" s="18" t="n"/>
       <c r="CW23" s="18" t="n"/>
       <c r="CX23" s="18" t="n"/>
-      <c r="CY23" s="18" t="n"/>
+      <c r="CY23" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CZ23" s="18" t="n"/>
       <c r="DA23" s="18" t="n"/>
       <c r="DB23" s="18" t="n"/>
@@ -13744,7 +13748,9 @@
       <c r="CX31" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CY31" s="18" t="n"/>
+      <c r="CY31" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CZ31" s="18" t="n"/>
       <c r="DA31" s="18" t="n"/>
       <c r="DB31" s="18" t="n"/>
@@ -16280,7 +16286,9 @@
       <c r="CV40" s="18" t="n"/>
       <c r="CW40" s="18" t="n"/>
       <c r="CX40" s="18" t="n"/>
-      <c r="CY40" s="18" t="n"/>
+      <c r="CY40" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="CZ40" s="18" t="n"/>
       <c r="DA40" s="18" t="n"/>
       <c r="DB40" s="18" t="n"/>
@@ -17651,7 +17659,9 @@
       <c r="CX45" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="CY45" s="18" t="n"/>
+      <c r="CY45" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CZ45" s="18" t="n"/>
       <c r="DA45" s="18" t="n"/>
       <c r="DB45" s="18" t="n"/>
@@ -24105,7 +24115,9 @@
       </c>
       <c r="CW68" s="18" t="n"/>
       <c r="CX68" s="18" t="n"/>
-      <c r="CY68" s="18" t="n"/>
+      <c r="CY68" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="CZ68" s="18" t="n"/>
       <c r="DA68" s="18" t="n"/>
       <c r="DB68" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-26 22:51 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8292,7 +8292,9 @@
       <c r="CW12" s="18" t="n"/>
       <c r="CX12" s="18" t="n"/>
       <c r="CY12" s="18" t="n"/>
-      <c r="CZ12" s="18" t="n"/>
+      <c r="CZ12" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DA12" s="18" t="n"/>
       <c r="DB12" s="18" t="n"/>
       <c r="DC12" s="18" t="n"/>
@@ -10877,7 +10879,9 @@
       </c>
       <c r="CX21" s="18" t="n"/>
       <c r="CY21" s="18" t="n"/>
-      <c r="CZ21" s="18" t="n"/>
+      <c r="CZ21" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DA21" s="18" t="n"/>
       <c r="DB21" s="18" t="n"/>
       <c r="DC21" s="18" t="n"/>
@@ -13751,7 +13755,9 @@
       <c r="CY31" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="CZ31" s="18" t="n"/>
+      <c r="CZ31" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DA31" s="18" t="n"/>
       <c r="DB31" s="18" t="n"/>
       <c r="DC31" s="18" t="n"/>
@@ -17662,7 +17668,9 @@
       <c r="CY45" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="CZ45" s="18" t="n"/>
+      <c r="CZ45" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DA45" s="18" t="n"/>
       <c r="DB45" s="18" t="n"/>
       <c r="DC45" s="18" t="n"/>
@@ -23563,7 +23571,9 @@
         <v>2</v>
       </c>
       <c r="CY66" s="18" t="n"/>
-      <c r="CZ66" s="18" t="n"/>
+      <c r="CZ66" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DA66" s="18" t="n"/>
       <c r="DB66" s="18" t="n"/>
       <c r="DC66" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-26 22:54 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -10883,7 +10883,9 @@
         <v>0.5</v>
       </c>
       <c r="DA21" s="18" t="n"/>
-      <c r="DB21" s="18" t="n"/>
+      <c r="DB21" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DC21" s="18" t="n"/>
       <c r="DD21" s="18" t="n"/>
       <c r="DE21" s="19" t="n"/>
@@ -11468,7 +11470,9 @@
       </c>
       <c r="CZ23" s="18" t="n"/>
       <c r="DA23" s="18" t="n"/>
-      <c r="DB23" s="18" t="n"/>
+      <c r="DB23" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DC23" s="18" t="n"/>
       <c r="DD23" s="18" t="n"/>
       <c r="DE23" s="19" t="n"/>
@@ -13759,7 +13763,9 @@
         <v>2</v>
       </c>
       <c r="DA31" s="18" t="n"/>
-      <c r="DB31" s="18" t="n"/>
+      <c r="DB31" s="18" t="n">
+        <v>2.5</v>
+      </c>
       <c r="DC31" s="18" t="n"/>
       <c r="DD31" s="18" t="n"/>
       <c r="DE31" s="19" t="n"/>
@@ -23575,7 +23581,9 @@
         <v>3</v>
       </c>
       <c r="DA66" s="18" t="n"/>
-      <c r="DB66" s="18" t="n"/>
+      <c r="DB66" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DC66" s="18" t="n"/>
       <c r="DD66" s="18" t="n"/>
       <c r="DE66" s="19" t="n"/>
@@ -26087,7 +26095,9 @@
       <c r="CY75" s="18" t="n"/>
       <c r="CZ75" s="18" t="n"/>
       <c r="DA75" s="18" t="n"/>
-      <c r="DB75" s="18" t="n"/>
+      <c r="DB75" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DC75" s="18" t="n"/>
       <c r="DD75" s="18" t="n"/>
       <c r="DE75" s="19" t="n"/>
@@ -26404,7 +26414,9 @@
       <c r="CY76" s="18" t="n"/>
       <c r="CZ76" s="18" t="n"/>
       <c r="DA76" s="18" t="n"/>
-      <c r="DB76" s="18" t="n"/>
+      <c r="DB76" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DC76" s="18" t="n"/>
       <c r="DD76" s="18" t="n"/>
       <c r="DE76" s="19" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-27 22:00 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8003,7 +8003,9 @@
       <c r="CZ11" s="18" t="n"/>
       <c r="DA11" s="18" t="n"/>
       <c r="DB11" s="18" t="n"/>
-      <c r="DC11" s="18" t="n"/>
+      <c r="DC11" s="18" t="n">
+        <v>1.25</v>
+      </c>
       <c r="DD11" s="18" t="n"/>
       <c r="DE11" s="19" t="n"/>
       <c r="DF11" s="18" t="n"/>
@@ -10886,7 +10888,9 @@
       <c r="DB21" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="DC21" s="18" t="n"/>
+      <c r="DC21" s="18" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DD21" s="18" t="n"/>
       <c r="DE21" s="19" t="n"/>
       <c r="DF21" s="18" t="n"/>
@@ -11473,7 +11477,9 @@
       <c r="DB23" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="DC23" s="18" t="n"/>
+      <c r="DC23" s="18" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DD23" s="18" t="n"/>
       <c r="DE23" s="19" t="n"/>
       <c r="DF23" s="18" t="n"/>
@@ -13766,7 +13772,9 @@
       <c r="DB31" s="18" t="n">
         <v>2.5</v>
       </c>
-      <c r="DC31" s="18" t="n"/>
+      <c r="DC31" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DD31" s="18" t="n"/>
       <c r="DE31" s="19" t="n"/>
       <c r="DF31" s="18" t="n"/>
@@ -14038,7 +14046,9 @@
       <c r="CZ32" s="18" t="n"/>
       <c r="DA32" s="18" t="n"/>
       <c r="DB32" s="18" t="n"/>
-      <c r="DC32" s="18" t="n"/>
+      <c r="DC32" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DD32" s="18" t="n"/>
       <c r="DE32" s="19" t="n"/>
       <c r="DF32" s="18" t="n"/>
@@ -14392,7 +14402,9 @@
       <c r="CZ33" s="18" t="n"/>
       <c r="DA33" s="18" t="n"/>
       <c r="DB33" s="18" t="n"/>
-      <c r="DC33" s="18" t="n"/>
+      <c r="DC33" s="18" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DD33" s="18" t="n"/>
       <c r="DE33" s="19" t="n"/>
       <c r="DF33" s="18" t="n"/>
@@ -23584,7 +23596,9 @@
       <c r="DB66" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="DC66" s="18" t="n"/>
+      <c r="DC66" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DD66" s="18" t="n"/>
       <c r="DE66" s="19" t="n"/>
       <c r="DF66" s="18" t="n"/>
@@ -26098,7 +26112,9 @@
       <c r="DB75" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="DC75" s="18" t="n"/>
+      <c r="DC75" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DD75" s="18" t="n"/>
       <c r="DE75" s="19" t="n"/>
       <c r="DF75" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-28 17:50 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8600,7 +8600,9 @@
       <c r="DA13" s="18" t="n"/>
       <c r="DB13" s="18" t="n"/>
       <c r="DC13" s="18" t="n"/>
-      <c r="DD13" s="18" t="n"/>
+      <c r="DD13" s="18" t="n">
+        <v>5</v>
+      </c>
       <c r="DE13" s="19" t="n"/>
       <c r="DF13" s="18" t="n"/>
       <c r="DG13" s="18" t="n"/>
@@ -17404,7 +17406,9 @@
       <c r="DA44" s="18" t="n"/>
       <c r="DB44" s="18" t="n"/>
       <c r="DC44" s="18" t="n"/>
-      <c r="DD44" s="18" t="n"/>
+      <c r="DD44" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DE44" s="19" t="n"/>
       <c r="DF44" s="18" t="n"/>
       <c r="DG44" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-05-28 21:59 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -17696,7 +17696,9 @@
       <c r="DA45" s="18" t="n"/>
       <c r="DB45" s="18" t="n"/>
       <c r="DC45" s="18" t="n"/>
-      <c r="DD45" s="18" t="n"/>
+      <c r="DD45" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DE45" s="19" t="n"/>
       <c r="DF45" s="18" t="n"/>
       <c r="DG45" s="18" t="n"/>
@@ -23603,7 +23605,9 @@
       <c r="DC66" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="DD66" s="18" t="n"/>
+      <c r="DD66" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DE66" s="19" t="n"/>
       <c r="DF66" s="18" t="n"/>
       <c r="DG66" s="18" t="n"/>
@@ -24158,7 +24162,9 @@
       <c r="DA68" s="18" t="n"/>
       <c r="DB68" s="18" t="n"/>
       <c r="DC68" s="18" t="n"/>
-      <c r="DD68" s="18" t="n"/>
+      <c r="DD68" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DE68" s="19" t="n"/>
       <c r="DF68" s="18" t="n"/>
       <c r="DG68" s="18" t="n"/>
@@ -26438,7 +26444,9 @@
         <v>1</v>
       </c>
       <c r="DC76" s="18" t="n"/>
-      <c r="DD76" s="18" t="n"/>
+      <c r="DD76" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DE76" s="19" t="n"/>
       <c r="DF76" s="18" t="n"/>
       <c r="DG76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-01 19:20 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -11483,7 +11483,9 @@
         <v>0.25</v>
       </c>
       <c r="DD23" s="18" t="n"/>
-      <c r="DE23" s="19" t="n"/>
+      <c r="DE23" s="19" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DF23" s="18" t="n"/>
       <c r="DG23" s="18" t="n"/>
       <c r="DH23" s="18" t="n"/>
@@ -13778,7 +13780,9 @@
         <v>1.5</v>
       </c>
       <c r="DD31" s="18" t="n"/>
-      <c r="DE31" s="19" t="n"/>
+      <c r="DE31" s="19" t="n">
+        <v>4</v>
+      </c>
       <c r="DF31" s="18" t="n"/>
       <c r="DG31" s="18" t="n"/>
       <c r="DH31" s="18" t="n"/>
@@ -18799,7 +18803,9 @@
       <c r="DB49" s="18" t="n"/>
       <c r="DC49" s="18" t="n"/>
       <c r="DD49" s="18" t="n"/>
-      <c r="DE49" s="19" t="n"/>
+      <c r="DE49" s="19" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DF49" s="18" t="n"/>
       <c r="DG49" s="18" t="n"/>
       <c r="DH49" s="18" t="n"/>
@@ -23608,7 +23614,9 @@
       <c r="DD66" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="DE66" s="19" t="n"/>
+      <c r="DE66" s="19" t="n">
+        <v>2</v>
+      </c>
       <c r="DF66" s="18" t="n"/>
       <c r="DG66" s="18" t="n"/>
       <c r="DH66" s="18" t="n"/>
@@ -26126,7 +26134,9 @@
         <v>3</v>
       </c>
       <c r="DD75" s="18" t="n"/>
-      <c r="DE75" s="19" t="n"/>
+      <c r="DE75" s="19" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DF75" s="18" t="n"/>
       <c r="DG75" s="18" t="n"/>
       <c r="DH75" s="18" t="n"/>
@@ -26447,7 +26457,9 @@
       <c r="DD76" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="DE76" s="19" t="n"/>
+      <c r="DE76" s="19" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DF76" s="18" t="n"/>
       <c r="DG76" s="18" t="n"/>
       <c r="DH76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-01 19:21 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -13783,7 +13783,9 @@
       <c r="DE31" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="DF31" s="18" t="n"/>
+      <c r="DF31" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DG31" s="18" t="n"/>
       <c r="DH31" s="18" t="n"/>
       <c r="DI31" s="18" t="n"/>
@@ -24174,7 +24176,9 @@
         <v>1</v>
       </c>
       <c r="DE68" s="19" t="n"/>
-      <c r="DF68" s="18" t="n"/>
+      <c r="DF68" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DG68" s="18" t="n"/>
       <c r="DH68" s="18" t="n"/>
       <c r="DI68" s="18" t="n"/>
@@ -26460,7 +26464,9 @@
       <c r="DE76" s="19" t="n">
         <v>0.5</v>
       </c>
-      <c r="DF76" s="18" t="n"/>
+      <c r="DF76" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DG76" s="18" t="n"/>
       <c r="DH76" s="18" t="n"/>
       <c r="DI76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-01 21:59 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -13784,7 +13784,7 @@
         <v>4</v>
       </c>
       <c r="DF31" s="18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="DG31" s="18" t="n"/>
       <c r="DH31" s="18" t="n"/>
@@ -23619,7 +23619,9 @@
       <c r="DE66" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="DF66" s="18" t="n"/>
+      <c r="DF66" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DG66" s="18" t="n"/>
       <c r="DH66" s="18" t="n"/>
       <c r="DI66" s="18" t="n"/>
@@ -24176,9 +24178,7 @@
         <v>1</v>
       </c>
       <c r="DE68" s="19" t="n"/>
-      <c r="DF68" s="18" t="n">
-        <v>2</v>
-      </c>
+      <c r="DF68" s="18" t="n"/>
       <c r="DG68" s="18" t="n"/>
       <c r="DH68" s="18" t="n"/>
       <c r="DI68" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-03 14:52 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8009,7 +8009,9 @@
       <c r="DD11" s="18" t="n"/>
       <c r="DE11" s="19" t="n"/>
       <c r="DF11" s="18" t="n"/>
-      <c r="DG11" s="18" t="n"/>
+      <c r="DG11" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DH11" s="18" t="n"/>
       <c r="DI11" s="18" t="n"/>
       <c r="DJ11" s="18" t="n"/>
@@ -13786,7 +13788,9 @@
       <c r="DF31" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="DG31" s="18" t="n"/>
+      <c r="DG31" s="18" t="n">
+        <v>4</v>
+      </c>
       <c r="DH31" s="18" t="n"/>
       <c r="DI31" s="18" t="n"/>
       <c r="DJ31" s="18" t="n"/>
@@ -23622,7 +23626,9 @@
       <c r="DF66" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="DG66" s="18" t="n"/>
+      <c r="DG66" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DH66" s="18" t="n"/>
       <c r="DI66" s="18" t="n"/>
       <c r="DJ66" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-03 17:48 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -10899,7 +10899,9 @@
       <c r="DE21" s="19" t="n"/>
       <c r="DF21" s="18" t="n"/>
       <c r="DG21" s="18" t="n"/>
-      <c r="DH21" s="18" t="n"/>
+      <c r="DH21" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DI21" s="18" t="n"/>
       <c r="DJ21" s="18" t="n"/>
       <c r="DK21" s="18" t="n"/>
@@ -13791,7 +13793,9 @@
       <c r="DG31" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="DH31" s="18" t="n"/>
+      <c r="DH31" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DI31" s="18" t="n"/>
       <c r="DJ31" s="18" t="n"/>
       <c r="DK31" s="18" t="n"/>
@@ -23629,7 +23633,9 @@
       <c r="DG66" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="DH66" s="18" t="n"/>
+      <c r="DH66" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DI66" s="18" t="n"/>
       <c r="DJ66" s="18" t="n"/>
       <c r="DK66" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-09 14:11 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -13794,7 +13794,7 @@
         <v>4</v>
       </c>
       <c r="DH31" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="DI31" s="18" t="n"/>
       <c r="DJ31" s="18" t="n"/>
@@ -23634,7 +23634,7 @@
         <v>3</v>
       </c>
       <c r="DH66" s="18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="DI66" s="18" t="n"/>
       <c r="DJ66" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-09 14:12 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8307,7 +8307,9 @@
       <c r="DF12" s="18" t="n"/>
       <c r="DG12" s="18" t="n"/>
       <c r="DH12" s="18" t="n"/>
-      <c r="DI12" s="18" t="n"/>
+      <c r="DI12" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DJ12" s="18" t="n"/>
       <c r="DK12" s="18" t="n"/>
       <c r="DL12" s="18" t="n"/>
@@ -10902,7 +10904,9 @@
       <c r="DH21" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="DI21" s="18" t="n"/>
+      <c r="DI21" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DJ21" s="18" t="n"/>
       <c r="DK21" s="18" t="n"/>
       <c r="DL21" s="18" t="n"/>
@@ -13796,7 +13800,9 @@
       <c r="DH31" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="DI31" s="18" t="n"/>
+      <c r="DI31" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DJ31" s="18" t="n"/>
       <c r="DK31" s="18" t="n"/>
       <c r="DL31" s="18" t="n"/>
@@ -23636,7 +23642,9 @@
       <c r="DH66" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="DI66" s="18" t="n"/>
+      <c r="DI66" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DJ66" s="18" t="n"/>
       <c r="DK66" s="18" t="n"/>
       <c r="DL66" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-09 14:15 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8310,7 +8310,9 @@
       <c r="DI12" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="DJ12" s="18" t="n"/>
+      <c r="DJ12" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DK12" s="18" t="n"/>
       <c r="DL12" s="18" t="n"/>
       <c r="DM12" s="18" t="n"/>
@@ -13803,7 +13805,9 @@
       <c r="DI31" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="DJ31" s="18" t="n"/>
+      <c r="DJ31" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DK31" s="18" t="n"/>
       <c r="DL31" s="18" t="n"/>
       <c r="DM31" s="18" t="n"/>
@@ -24202,7 +24206,9 @@
       <c r="DG68" s="18" t="n"/>
       <c r="DH68" s="18" t="n"/>
       <c r="DI68" s="18" t="n"/>
-      <c r="DJ68" s="18" t="n"/>
+      <c r="DJ68" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DK68" s="18" t="n"/>
       <c r="DL68" s="18" t="n"/>
       <c r="DM68" s="18" t="n"/>
@@ -26490,7 +26496,9 @@
       <c r="DG76" s="18" t="n"/>
       <c r="DH76" s="18" t="n"/>
       <c r="DI76" s="18" t="n"/>
-      <c r="DJ76" s="18" t="n"/>
+      <c r="DJ76" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DK76" s="18" t="n"/>
       <c r="DL76" s="18" t="n"/>
       <c r="DM76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-09 14:16 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8015,7 +8015,9 @@
       <c r="DH11" s="18" t="n"/>
       <c r="DI11" s="18" t="n"/>
       <c r="DJ11" s="18" t="n"/>
-      <c r="DK11" s="18" t="n"/>
+      <c r="DK11" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DL11" s="18" t="n"/>
       <c r="DM11" s="18" t="n"/>
       <c r="DN11" s="18" t="n"/>
@@ -8313,7 +8315,9 @@
       <c r="DJ12" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="DK12" s="18" t="n"/>
+      <c r="DK12" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DL12" s="18" t="n"/>
       <c r="DM12" s="18" t="n"/>
       <c r="DN12" s="18" t="n"/>
@@ -13808,7 +13812,9 @@
       <c r="DJ31" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="DK31" s="18" t="n"/>
+      <c r="DK31" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DL31" s="18" t="n"/>
       <c r="DM31" s="18" t="n"/>
       <c r="DN31" s="18" t="n"/>
@@ -23650,7 +23656,9 @@
         <v>3</v>
       </c>
       <c r="DJ66" s="18" t="n"/>
-      <c r="DK66" s="18" t="n"/>
+      <c r="DK66" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DL66" s="18" t="n"/>
       <c r="DM66" s="18" t="n"/>
       <c r="DN66" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-11 18:04 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -10915,7 +10915,9 @@
       </c>
       <c r="DJ21" s="18" t="n"/>
       <c r="DK21" s="18" t="n"/>
-      <c r="DL21" s="18" t="n"/>
+      <c r="DL21" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DM21" s="18" t="n"/>
       <c r="DN21" s="18" t="n"/>
       <c r="DO21" s="18" t="n"/>
@@ -11506,7 +11508,9 @@
       <c r="DI23" s="18" t="n"/>
       <c r="DJ23" s="18" t="n"/>
       <c r="DK23" s="18" t="n"/>
-      <c r="DL23" s="18" t="n"/>
+      <c r="DL23" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DM23" s="18" t="n"/>
       <c r="DN23" s="18" t="n"/>
       <c r="DO23" s="18" t="n"/>
@@ -13815,7 +13819,9 @@
       <c r="DK31" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="DL31" s="18" t="n"/>
+      <c r="DL31" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DM31" s="18" t="n"/>
       <c r="DN31" s="18" t="n"/>
       <c r="DO31" s="18" t="n"/>
@@ -23659,7 +23665,9 @@
       <c r="DK66" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="DL66" s="18" t="n"/>
+      <c r="DL66" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DM66" s="18" t="n"/>
       <c r="DN66" s="18" t="n"/>
       <c r="DO66" s="18" t="n"/>
@@ -26181,7 +26189,9 @@
       <c r="DI75" s="18" t="n"/>
       <c r="DJ75" s="18" t="n"/>
       <c r="DK75" s="18" t="n"/>
-      <c r="DL75" s="18" t="n"/>
+      <c r="DL75" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DM75" s="18" t="n"/>
       <c r="DN75" s="18" t="n"/>
       <c r="DO75" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-11 18:06 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -7667,7 +7667,9 @@
       <c r="DJ10" s="18" t="n"/>
       <c r="DK10" s="18" t="n"/>
       <c r="DL10" s="18" t="n"/>
-      <c r="DM10" s="18" t="n"/>
+      <c r="DM10" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DN10" s="18" t="n"/>
       <c r="DO10" s="18" t="n"/>
       <c r="DP10" s="18" t="n"/>
@@ -10918,7 +10920,9 @@
       <c r="DL21" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="DM21" s="18" t="n"/>
+      <c r="DM21" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DN21" s="18" t="n"/>
       <c r="DO21" s="18" t="n"/>
       <c r="DP21" s="18" t="n"/>
@@ -13822,7 +13826,9 @@
       <c r="DL31" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="DM31" s="18" t="n"/>
+      <c r="DM31" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DN31" s="18" t="n"/>
       <c r="DO31" s="18" t="n"/>
       <c r="DP31" s="18" t="n"/>
@@ -24227,7 +24233,9 @@
       </c>
       <c r="DK68" s="18" t="n"/>
       <c r="DL68" s="18" t="n"/>
-      <c r="DM68" s="18" t="n"/>
+      <c r="DM68" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DN68" s="18" t="n"/>
       <c r="DO68" s="18" t="n"/>
       <c r="DP68" s="18" t="n"/>
@@ -25041,7 +25049,9 @@
       <c r="DJ71" s="18" t="n"/>
       <c r="DK71" s="18" t="n"/>
       <c r="DL71" s="18" t="n"/>
-      <c r="DM71" s="18" t="n"/>
+      <c r="DM71" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DN71" s="18" t="n"/>
       <c r="DO71" s="18" t="n"/>
       <c r="DP71" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-11 19:14 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -7670,7 +7670,9 @@
       <c r="DM10" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="DN10" s="18" t="n"/>
+      <c r="DN10" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DO10" s="18" t="n"/>
       <c r="DP10" s="18" t="n"/>
       <c r="DQ10" s="18" t="n"/>
@@ -9744,7 +9746,9 @@
       <c r="DK17" s="18" t="n"/>
       <c r="DL17" s="18" t="n"/>
       <c r="DM17" s="18" t="n"/>
-      <c r="DN17" s="18" t="n"/>
+      <c r="DN17" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DO17" s="18" t="n"/>
       <c r="DP17" s="18" t="n"/>
       <c r="DQ17" s="18" t="n"/>
@@ -13829,7 +13833,9 @@
       <c r="DM31" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="DN31" s="18" t="n"/>
+      <c r="DN31" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DO31" s="18" t="n"/>
       <c r="DP31" s="18" t="n"/>
       <c r="DQ31" s="18" t="n"/>
@@ -14459,7 +14465,9 @@
       <c r="DK33" s="18" t="n"/>
       <c r="DL33" s="18" t="n"/>
       <c r="DM33" s="18" t="n"/>
-      <c r="DN33" s="18" t="n"/>
+      <c r="DN33" s="18" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DO33" s="18" t="n"/>
       <c r="DP33" s="18" t="n"/>
       <c r="DQ33" s="18" t="n"/>
@@ -23675,7 +23683,9 @@
         <v>3</v>
       </c>
       <c r="DM66" s="18" t="n"/>
-      <c r="DN66" s="18" t="n"/>
+      <c r="DN66" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DO66" s="18" t="n"/>
       <c r="DP66" s="18" t="n"/>
       <c r="DQ66" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-11 21:37 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8324,7 +8324,9 @@
       </c>
       <c r="DL12" s="18" t="n"/>
       <c r="DM12" s="18" t="n"/>
-      <c r="DN12" s="18" t="n"/>
+      <c r="DN12" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DO12" s="18" t="n"/>
       <c r="DP12" s="18" t="n"/>
       <c r="DQ12" s="18" t="n"/>
@@ -26540,7 +26542,9 @@
       <c r="DK76" s="18" t="n"/>
       <c r="DL76" s="18" t="n"/>
       <c r="DM76" s="18" t="n"/>
-      <c r="DN76" s="18" t="n"/>
+      <c r="DN76" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DO76" s="18" t="n"/>
       <c r="DP76" s="18" t="n"/>
       <c r="DQ76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-12 18:54 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -9193,7 +9193,9 @@
       <c r="DL15" s="18" t="n"/>
       <c r="DM15" s="18" t="n"/>
       <c r="DN15" s="18" t="n"/>
-      <c r="DO15" s="18" t="n"/>
+      <c r="DO15" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DP15" s="18" t="n"/>
       <c r="DQ15" s="18" t="n"/>
       <c r="DR15" s="18" t="n"/>
@@ -9751,7 +9753,9 @@
       <c r="DN17" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="DO17" s="18" t="n"/>
+      <c r="DO17" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DP17" s="18" t="n"/>
       <c r="DQ17" s="18" t="n"/>
       <c r="DR17" s="18" t="n"/>
@@ -11523,7 +11527,9 @@
       </c>
       <c r="DM23" s="18" t="n"/>
       <c r="DN23" s="18" t="n"/>
-      <c r="DO23" s="18" t="n"/>
+      <c r="DO23" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DP23" s="18" t="n"/>
       <c r="DQ23" s="18" t="n"/>
       <c r="DR23" s="18" t="n"/>
@@ -23688,7 +23694,9 @@
       <c r="DN66" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="DO66" s="18" t="n"/>
+      <c r="DO66" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DP66" s="18" t="n"/>
       <c r="DQ66" s="18" t="n"/>
       <c r="DR66" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-12 21:38 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -10934,7 +10934,9 @@
         <v>0.5</v>
       </c>
       <c r="DN21" s="18" t="n"/>
-      <c r="DO21" s="18" t="n"/>
+      <c r="DO21" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DP21" s="18" t="n"/>
       <c r="DQ21" s="18" t="n"/>
       <c r="DR21" s="18" t="n"/>
@@ -13844,7 +13846,9 @@
       <c r="DN31" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="DO31" s="18" t="n"/>
+      <c r="DO31" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DP31" s="18" t="n"/>
       <c r="DQ31" s="18" t="n"/>
       <c r="DR31" s="18" t="n"/>
@@ -14476,7 +14480,9 @@
       <c r="DN33" s="18" t="n">
         <v>0.25</v>
       </c>
-      <c r="DO33" s="18" t="n"/>
+      <c r="DO33" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DP33" s="18" t="n"/>
       <c r="DQ33" s="18" t="n"/>
       <c r="DR33" s="18" t="n"/>
@@ -24257,7 +24263,9 @@
         <v>3</v>
       </c>
       <c r="DN68" s="18" t="n"/>
-      <c r="DO68" s="18" t="n"/>
+      <c r="DO68" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DP68" s="18" t="n"/>
       <c r="DQ68" s="18" t="n"/>
       <c r="DR68" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-15 22:44 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8026,7 +8026,9 @@
       <c r="DM11" s="18" t="n"/>
       <c r="DN11" s="18" t="n"/>
       <c r="DO11" s="18" t="n"/>
-      <c r="DP11" s="18" t="n"/>
+      <c r="DP11" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DQ11" s="18" t="n"/>
       <c r="DR11" s="18" t="n"/>
       <c r="DS11" s="18" t="n"/>
@@ -8328,7 +8330,9 @@
         <v>1</v>
       </c>
       <c r="DO12" s="18" t="n"/>
-      <c r="DP12" s="18" t="n"/>
+      <c r="DP12" s="18" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DQ12" s="18" t="n"/>
       <c r="DR12" s="18" t="n"/>
       <c r="DS12" s="18" t="n"/>
@@ -10937,7 +10941,9 @@
       <c r="DO21" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="DP21" s="18" t="n"/>
+      <c r="DP21" s="18" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DQ21" s="18" t="n"/>
       <c r="DR21" s="18" t="n"/>
       <c r="DS21" s="18" t="n"/>
@@ -11532,7 +11538,9 @@
       <c r="DO23" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="DP23" s="18" t="n"/>
+      <c r="DP23" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DQ23" s="18" t="n"/>
       <c r="DR23" s="18" t="n"/>
       <c r="DS23" s="18" t="n"/>
@@ -13849,7 +13857,9 @@
       <c r="DO31" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="DP31" s="18" t="n"/>
+      <c r="DP31" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DQ31" s="18" t="n"/>
       <c r="DR31" s="18" t="n"/>
       <c r="DS31" s="18" t="n"/>
@@ -24266,7 +24276,9 @@
       <c r="DO68" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="DP68" s="18" t="n"/>
+      <c r="DP68" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DQ68" s="18" t="n"/>
       <c r="DR68" s="18" t="n"/>
       <c r="DS68" s="18" t="n"/>
@@ -26562,7 +26574,9 @@
         <v>1</v>
       </c>
       <c r="DO76" s="18" t="n"/>
-      <c r="DP76" s="18" t="n"/>
+      <c r="DP76" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DQ76" s="18" t="n"/>
       <c r="DR76" s="18" t="n"/>
       <c r="DS76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-18 18:52 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -10944,7 +10944,9 @@
       <c r="DP21" s="18" t="n">
         <v>0.25</v>
       </c>
-      <c r="DQ21" s="18" t="n"/>
+      <c r="DQ21" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DR21" s="18" t="n"/>
       <c r="DS21" s="18" t="n"/>
       <c r="DT21" s="18" t="n"/>
@@ -23714,7 +23716,9 @@
         <v>0.5</v>
       </c>
       <c r="DP66" s="18" t="n"/>
-      <c r="DQ66" s="18" t="n"/>
+      <c r="DQ66" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DR66" s="18" t="n"/>
       <c r="DS66" s="18" t="n"/>
       <c r="DT66" s="18" t="n"/>
@@ -24279,7 +24283,9 @@
       <c r="DP68" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="DQ68" s="18" t="n"/>
+      <c r="DQ68" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DR68" s="18" t="n"/>
       <c r="DS68" s="18" t="n"/>
       <c r="DT68" s="18" t="n"/>
@@ -28544,7 +28550,9 @@
       <c r="DN83" s="18" t="n"/>
       <c r="DO83" s="18" t="n"/>
       <c r="DP83" s="18" t="n"/>
-      <c r="DQ83" s="18" t="n"/>
+      <c r="DQ83" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DR83" s="18" t="n"/>
       <c r="DS83" s="18" t="n"/>
       <c r="DT83" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-18 18:56 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -9762,7 +9762,9 @@
       </c>
       <c r="DP17" s="18" t="n"/>
       <c r="DQ17" s="18" t="n"/>
-      <c r="DR17" s="18" t="n"/>
+      <c r="DR17" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DS17" s="18" t="n"/>
       <c r="DT17" s="18" t="n"/>
       <c r="DU17" s="18" t="n"/>
@@ -10947,7 +10949,9 @@
       <c r="DQ21" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="DR21" s="18" t="n"/>
+      <c r="DR21" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DS21" s="18" t="n"/>
       <c r="DT21" s="18" t="n"/>
       <c r="DU21" s="18" t="n"/>
@@ -11544,7 +11548,9 @@
         <v>0.5</v>
       </c>
       <c r="DQ23" s="18" t="n"/>
-      <c r="DR23" s="18" t="n"/>
+      <c r="DR23" s="18" t="n">
+        <v>0.75</v>
+      </c>
       <c r="DS23" s="18" t="n"/>
       <c r="DT23" s="18" t="n"/>
       <c r="DU23" s="18" t="n"/>
@@ -13863,7 +13869,9 @@
         <v>1</v>
       </c>
       <c r="DQ31" s="18" t="n"/>
-      <c r="DR31" s="18" t="n"/>
+      <c r="DR31" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DS31" s="18" t="n"/>
       <c r="DT31" s="18" t="n"/>
       <c r="DU31" s="18" t="n"/>
@@ -15861,7 +15869,9 @@
       <c r="DO38" s="18" t="n"/>
       <c r="DP38" s="18" t="n"/>
       <c r="DQ38" s="18" t="n"/>
-      <c r="DR38" s="18" t="n"/>
+      <c r="DR38" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DS38" s="18" t="n"/>
       <c r="DT38" s="18" t="n"/>
       <c r="DU38" s="18" t="n"/>
@@ -23719,7 +23729,9 @@
       <c r="DQ66" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="DR66" s="18" t="n"/>
+      <c r="DR66" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DS66" s="18" t="n"/>
       <c r="DT66" s="18" t="n"/>
       <c r="DU66" s="18" t="n"/>
@@ -26584,7 +26596,9 @@
         <v>1.5</v>
       </c>
       <c r="DQ76" s="18" t="n"/>
-      <c r="DR76" s="18" t="n"/>
+      <c r="DR76" s="18" t="n">
+        <v>2.75</v>
+      </c>
       <c r="DS76" s="18" t="n"/>
       <c r="DT76" s="18" t="n"/>
       <c r="DU76" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-23 22:19 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -23733,7 +23733,9 @@
         <v>1</v>
       </c>
       <c r="DS66" s="18" t="n"/>
-      <c r="DT66" s="18" t="n"/>
+      <c r="DT66" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DU66" s="18" t="n"/>
       <c r="DV66" s="18" t="n"/>
       <c r="DW66" s="18" t="n"/>
@@ -28009,7 +28011,9 @@
       <c r="DQ81" s="18" t="n"/>
       <c r="DR81" s="18" t="n"/>
       <c r="DS81" s="18" t="n"/>
-      <c r="DT81" s="18" t="n"/>
+      <c r="DT81" s="18" t="n">
+        <v>6</v>
+      </c>
       <c r="DU81" s="18" t="n"/>
       <c r="DV81" s="18" t="n"/>
       <c r="DW81" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-23 22:21 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8033,7 +8033,9 @@
       <c r="DR11" s="18" t="n"/>
       <c r="DS11" s="18" t="n"/>
       <c r="DT11" s="18" t="n"/>
-      <c r="DU11" s="18" t="n"/>
+      <c r="DU11" s="18" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DV11" s="18" t="n"/>
       <c r="DW11" s="18" t="n"/>
       <c r="DX11" s="18" t="n"/>
@@ -13874,7 +13876,9 @@
       </c>
       <c r="DS31" s="18" t="n"/>
       <c r="DT31" s="18" t="n"/>
-      <c r="DU31" s="18" t="n"/>
+      <c r="DU31" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DV31" s="18" t="n"/>
       <c r="DW31" s="18" t="n"/>
       <c r="DX31" s="18" t="n"/>
@@ -20278,7 +20282,9 @@
       <c r="DR54" s="18" t="n"/>
       <c r="DS54" s="18" t="n"/>
       <c r="DT54" s="18" t="n"/>
-      <c r="DU54" s="18" t="n"/>
+      <c r="DU54" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DV54" s="18" t="n"/>
       <c r="DW54" s="18" t="n"/>
       <c r="DX54" s="18" t="n"/>
@@ -23736,7 +23742,9 @@
       <c r="DT66" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="DU66" s="18" t="n"/>
+      <c r="DU66" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DV66" s="18" t="n"/>
       <c r="DW66" s="18" t="n"/>
       <c r="DX66" s="18" t="n"/>
@@ -24303,7 +24311,9 @@
       <c r="DR68" s="18" t="n"/>
       <c r="DS68" s="18" t="n"/>
       <c r="DT68" s="18" t="n"/>
-      <c r="DU68" s="18" t="n"/>
+      <c r="DU68" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DV68" s="18" t="n"/>
       <c r="DW68" s="18" t="n"/>
       <c r="DX68" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-23 22:23 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -13879,7 +13879,9 @@
       <c r="DU31" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="DV31" s="18" t="n"/>
+      <c r="DV31" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DW31" s="18" t="n"/>
       <c r="DX31" s="18" t="n"/>
       <c r="DY31" s="18" t="n"/>
@@ -16968,7 +16970,9 @@
       <c r="DS42" s="18" t="n"/>
       <c r="DT42" s="18" t="n"/>
       <c r="DU42" s="18" t="n"/>
-      <c r="DV42" s="18" t="n"/>
+      <c r="DV42" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="DW42" s="18" t="n"/>
       <c r="DX42" s="18" t="n"/>
       <c r="DY42" s="18" t="n"/>
@@ -24314,7 +24318,9 @@
       <c r="DU68" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="DV68" s="18" t="n"/>
+      <c r="DV68" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DW68" s="18" t="n"/>
       <c r="DX68" s="18" t="n"/>
       <c r="DY68" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-25 16:59 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -11558,7 +11558,9 @@
       <c r="DU23" s="18" t="n"/>
       <c r="DV23" s="18" t="n"/>
       <c r="DW23" s="18" t="n"/>
-      <c r="DX23" s="18" t="n"/>
+      <c r="DX23" s="18" t="n">
+        <v>3.5</v>
+      </c>
       <c r="DY23" s="18" t="n"/>
       <c r="DZ23" s="18" t="n"/>
       <c r="EA23" s="19" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-25 17:02 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -13884,7 +13884,9 @@
       <c r="DV31" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="DW31" s="18" t="n"/>
+      <c r="DW31" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DX31" s="18" t="n"/>
       <c r="DY31" s="18" t="n"/>
       <c r="DZ31" s="18" t="n"/>
@@ -14518,7 +14520,9 @@
       <c r="DT33" s="18" t="n"/>
       <c r="DU33" s="18" t="n"/>
       <c r="DV33" s="18" t="n"/>
-      <c r="DW33" s="18" t="n"/>
+      <c r="DW33" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DX33" s="18" t="n"/>
       <c r="DY33" s="18" t="n"/>
       <c r="DZ33" s="18" t="n"/>
@@ -16975,7 +16979,9 @@
       <c r="DV42" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="DW42" s="18" t="n"/>
+      <c r="DW42" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DX42" s="18" t="n"/>
       <c r="DY42" s="18" t="n"/>
       <c r="DZ42" s="18" t="n"/>
@@ -23752,7 +23758,9 @@
         <v>2</v>
       </c>
       <c r="DV66" s="18" t="n"/>
-      <c r="DW66" s="18" t="n"/>
+      <c r="DW66" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DX66" s="18" t="n"/>
       <c r="DY66" s="18" t="n"/>
       <c r="DZ66" s="18" t="n"/>
@@ -26290,7 +26298,9 @@
       <c r="DT75" s="18" t="n"/>
       <c r="DU75" s="18" t="n"/>
       <c r="DV75" s="18" t="n"/>
-      <c r="DW75" s="18" t="n"/>
+      <c r="DW75" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DX75" s="18" t="n"/>
       <c r="DY75" s="18" t="n"/>
       <c r="DZ75" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-25 21:49 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8342,7 +8342,9 @@
       <c r="DU12" s="18" t="n"/>
       <c r="DV12" s="18" t="n"/>
       <c r="DW12" s="18" t="n"/>
-      <c r="DX12" s="18" t="n"/>
+      <c r="DX12" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DY12" s="18" t="n"/>
       <c r="DZ12" s="18" t="n"/>
       <c r="EA12" s="19" t="n"/>
@@ -11559,7 +11561,7 @@
       <c r="DV23" s="18" t="n"/>
       <c r="DW23" s="18" t="n"/>
       <c r="DX23" s="18" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="DY23" s="18" t="n"/>
       <c r="DZ23" s="18" t="n"/>
@@ -13887,7 +13889,9 @@
       <c r="DW31" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="DX31" s="18" t="n"/>
+      <c r="DX31" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DY31" s="18" t="n"/>
       <c r="DZ31" s="18" t="n"/>
       <c r="EA31" s="19" t="n"/>
@@ -14523,7 +14527,9 @@
       <c r="DW33" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="DX33" s="18" t="n"/>
+      <c r="DX33" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DY33" s="18" t="n"/>
       <c r="DZ33" s="18" t="n"/>
       <c r="EA33" s="19" t="n"/>
@@ -23761,7 +23767,9 @@
       <c r="DW66" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="DX66" s="18" t="n"/>
+      <c r="DX66" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DY66" s="18" t="n"/>
       <c r="DZ66" s="18" t="n"/>
       <c r="EA66" s="19" t="n"/>
@@ -24332,7 +24340,9 @@
         <v>2</v>
       </c>
       <c r="DW68" s="18" t="n"/>
-      <c r="DX68" s="18" t="n"/>
+      <c r="DX68" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="DY68" s="18" t="n"/>
       <c r="DZ68" s="18" t="n"/>
       <c r="EA68" s="19" t="n"/>
@@ -26634,7 +26644,9 @@
       <c r="DU76" s="18" t="n"/>
       <c r="DV76" s="18" t="n"/>
       <c r="DW76" s="18" t="n"/>
-      <c r="DX76" s="18" t="n"/>
+      <c r="DX76" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="DY76" s="18" t="n"/>
       <c r="DZ76" s="18" t="n"/>
       <c r="EA76" s="19" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-30 20:28 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -28058,7 +28058,9 @@
       <c r="DV81" s="18" t="n"/>
       <c r="DW81" s="18" t="n"/>
       <c r="DX81" s="18" t="n"/>
-      <c r="DY81" s="18" t="n"/>
+      <c r="DY81" s="18" t="n">
+        <v>8</v>
+      </c>
       <c r="DZ81" s="18" t="n"/>
       <c r="EA81" s="19" t="n"/>
       <c r="EB81" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-30 20:29 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -28062,7 +28062,9 @@
         <v>8</v>
       </c>
       <c r="DZ81" s="18" t="n"/>
-      <c r="EA81" s="19" t="n"/>
+      <c r="EA81" s="19" t="n">
+        <v>8</v>
+      </c>
       <c r="EB81" s="18" t="n"/>
       <c r="EC81" s="18" t="n"/>
       <c r="ED81" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-06-30 20:31 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8347,7 +8347,9 @@
       </c>
       <c r="DY12" s="18" t="n"/>
       <c r="DZ12" s="18" t="n"/>
-      <c r="EA12" s="19" t="n"/>
+      <c r="EA12" s="19" t="n">
+        <v>1</v>
+      </c>
       <c r="EB12" s="18" t="n"/>
       <c r="EC12" s="18" t="n"/>
       <c r="ED12" s="18" t="n"/>
@@ -10964,7 +10966,9 @@
       <c r="DX21" s="18" t="n"/>
       <c r="DY21" s="18" t="n"/>
       <c r="DZ21" s="18" t="n"/>
-      <c r="EA21" s="19" t="n"/>
+      <c r="EA21" s="19" t="n">
+        <v>1</v>
+      </c>
       <c r="EB21" s="18" t="n"/>
       <c r="EC21" s="18" t="n"/>
       <c r="ED21" s="18" t="n"/>
@@ -11565,7 +11569,9 @@
       </c>
       <c r="DY23" s="18" t="n"/>
       <c r="DZ23" s="18" t="n"/>
-      <c r="EA23" s="19" t="n"/>
+      <c r="EA23" s="19" t="n">
+        <v>1</v>
+      </c>
       <c r="EB23" s="18" t="n"/>
       <c r="EC23" s="18" t="n"/>
       <c r="ED23" s="18" t="n"/>
@@ -13894,7 +13900,9 @@
       </c>
       <c r="DY31" s="18" t="n"/>
       <c r="DZ31" s="18" t="n"/>
-      <c r="EA31" s="19" t="n"/>
+      <c r="EA31" s="19" t="n">
+        <v>1</v>
+      </c>
       <c r="EB31" s="18" t="n"/>
       <c r="EC31" s="18" t="n"/>
       <c r="ED31" s="18" t="n"/>
@@ -16991,7 +16999,9 @@
       <c r="DX42" s="18" t="n"/>
       <c r="DY42" s="18" t="n"/>
       <c r="DZ42" s="18" t="n"/>
-      <c r="EA42" s="19" t="n"/>
+      <c r="EA42" s="19" t="n">
+        <v>1</v>
+      </c>
       <c r="EB42" s="18" t="n"/>
       <c r="EC42" s="18" t="n"/>
       <c r="ED42" s="18" t="n"/>
@@ -23772,7 +23782,9 @@
       </c>
       <c r="DY66" s="18" t="n"/>
       <c r="DZ66" s="18" t="n"/>
-      <c r="EA66" s="19" t="n"/>
+      <c r="EA66" s="19" t="n">
+        <v>1</v>
+      </c>
       <c r="EB66" s="18" t="n"/>
       <c r="EC66" s="18" t="n"/>
       <c r="ED66" s="18" t="n"/>
@@ -27204,7 +27216,9 @@
       <c r="DX78" s="18" t="n"/>
       <c r="DY78" s="18" t="n"/>
       <c r="DZ78" s="18" t="n"/>
-      <c r="EA78" s="19" t="n"/>
+      <c r="EA78" s="19" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EB78" s="18" t="n"/>
       <c r="EC78" s="18" t="n"/>
       <c r="ED78" s="18" t="n"/>
@@ -28064,9 +28078,7 @@
       <c r="DZ81" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="EA81" s="19" t="n">
-        <v>8</v>
-      </c>
+      <c r="EA81" s="19" t="n"/>
       <c r="EB81" s="18" t="n"/>
       <c r="EC81" s="18" t="n"/>
       <c r="ED81" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-01 14:21 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -10967,7 +10967,7 @@
       <c r="DY21" s="18" t="n"/>
       <c r="DZ21" s="18" t="n"/>
       <c r="EA21" s="19" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="EB21" s="18" t="n"/>
       <c r="EC21" s="18" t="n"/>
@@ -13901,7 +13901,7 @@
       <c r="DY31" s="18" t="n"/>
       <c r="DZ31" s="18" t="n"/>
       <c r="EA31" s="19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="EB31" s="18" t="n"/>
       <c r="EC31" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-01 14:22 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -10969,7 +10969,9 @@
       <c r="EA21" s="19" t="n">
         <v>0.5</v>
       </c>
-      <c r="EB21" s="18" t="n"/>
+      <c r="EB21" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EC21" s="18" t="n"/>
       <c r="ED21" s="18" t="n"/>
       <c r="EE21" s="18" t="n"/>
@@ -13903,7 +13905,9 @@
       <c r="EA31" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="EB31" s="18" t="n"/>
+      <c r="EB31" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EC31" s="18" t="n"/>
       <c r="ED31" s="18" t="n"/>
       <c r="EE31" s="18" t="n"/>
@@ -19216,7 +19220,9 @@
       <c r="DY50" s="18" t="n"/>
       <c r="DZ50" s="18" t="n"/>
       <c r="EA50" s="19" t="n"/>
-      <c r="EB50" s="18" t="n"/>
+      <c r="EB50" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EC50" s="18" t="n"/>
       <c r="ED50" s="18" t="n"/>
       <c r="EE50" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-01 19:13 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -15911,7 +15911,9 @@
       <c r="DY38" s="18" t="n"/>
       <c r="DZ38" s="18" t="n"/>
       <c r="EA38" s="19" t="n"/>
-      <c r="EB38" s="18" t="n"/>
+      <c r="EB38" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EC38" s="18" t="n"/>
       <c r="ED38" s="18" t="n"/>
       <c r="EE38" s="18" t="n"/>
@@ -26333,7 +26335,9 @@
       <c r="DY75" s="18" t="n"/>
       <c r="DZ75" s="18" t="n"/>
       <c r="EA75" s="19" t="n"/>
-      <c r="EB75" s="18" t="n"/>
+      <c r="EB75" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EC75" s="18" t="n"/>
       <c r="ED75" s="18" t="n"/>
       <c r="EE75" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-02 13:07 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -13906,7 +13906,7 @@
         <v>3</v>
       </c>
       <c r="EB31" s="18" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="EC31" s="18" t="n"/>
       <c r="ED31" s="18" t="n"/>
@@ -14181,7 +14181,9 @@
       <c r="DY32" s="18" t="n"/>
       <c r="DZ32" s="18" t="n"/>
       <c r="EA32" s="19" t="n"/>
-      <c r="EB32" s="18" t="n"/>
+      <c r="EB32" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EC32" s="18" t="n"/>
       <c r="ED32" s="18" t="n"/>
       <c r="EE32" s="18" t="n"/>
@@ -24366,7 +24368,9 @@
       <c r="DY68" s="18" t="n"/>
       <c r="DZ68" s="18" t="n"/>
       <c r="EA68" s="19" t="n"/>
-      <c r="EB68" s="18" t="n"/>
+      <c r="EB68" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EC68" s="18" t="n"/>
       <c r="ED68" s="18" t="n"/>
       <c r="EE68" s="18" t="n"/>
@@ -26336,7 +26340,7 @@
       <c r="DZ75" s="18" t="n"/>
       <c r="EA75" s="19" t="n"/>
       <c r="EB75" s="18" t="n">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="EC75" s="18" t="n"/>
       <c r="ED75" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-02 14:34 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8043,7 +8043,9 @@
       <c r="DZ11" s="18" t="n"/>
       <c r="EA11" s="19" t="n"/>
       <c r="EB11" s="18" t="n"/>
-      <c r="EC11" s="18" t="n"/>
+      <c r="EC11" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="ED11" s="18" t="n"/>
       <c r="EE11" s="18" t="n"/>
       <c r="EF11" s="18" t="n"/>
@@ -13908,7 +13910,9 @@
       <c r="EB31" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="EC31" s="18" t="n"/>
+      <c r="EC31" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="ED31" s="18" t="n"/>
       <c r="EE31" s="18" t="n"/>
       <c r="EF31" s="18" t="n"/>
@@ -27234,7 +27238,9 @@
         <v>0.5</v>
       </c>
       <c r="EB78" s="18" t="n"/>
-      <c r="EC78" s="18" t="n"/>
+      <c r="EC78" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="ED78" s="18" t="n"/>
       <c r="EE78" s="18" t="n"/>
       <c r="EF78" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-06 13:37 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -17017,7 +17017,9 @@
       <c r="EB42" s="18" t="n"/>
       <c r="EC42" s="18" t="n"/>
       <c r="ED42" s="18" t="n"/>
-      <c r="EE42" s="18" t="n"/>
+      <c r="EE42" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="EF42" s="18" t="n"/>
       <c r="EG42" s="18" t="n"/>
       <c r="EH42" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-06 13:38 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -27793,7 +27793,9 @@
       <c r="EA80" s="19" t="n"/>
       <c r="EB80" s="18" t="n"/>
       <c r="EC80" s="18" t="n"/>
-      <c r="ED80" s="18" t="n"/>
+      <c r="ED80" s="18" t="n">
+        <v>8</v>
+      </c>
       <c r="EE80" s="18" t="n"/>
       <c r="EF80" s="18" t="n"/>
       <c r="EG80" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-06 20:36 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8047,7 +8047,9 @@
         <v>1</v>
       </c>
       <c r="ED11" s="18" t="n"/>
-      <c r="EE11" s="18" t="n"/>
+      <c r="EE11" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="EF11" s="18" t="n"/>
       <c r="EG11" s="18" t="n"/>
       <c r="EH11" s="18" t="n"/>
@@ -10976,7 +10978,9 @@
       </c>
       <c r="EC21" s="18" t="n"/>
       <c r="ED21" s="18" t="n"/>
-      <c r="EE21" s="18" t="n"/>
+      <c r="EE21" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EF21" s="18" t="n"/>
       <c r="EG21" s="18" t="n"/>
       <c r="EH21" s="18" t="n"/>
@@ -11579,7 +11583,9 @@
       <c r="EB23" s="18" t="n"/>
       <c r="EC23" s="18" t="n"/>
       <c r="ED23" s="18" t="n"/>
-      <c r="EE23" s="18" t="n"/>
+      <c r="EE23" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EF23" s="18" t="n"/>
       <c r="EG23" s="18" t="n"/>
       <c r="EH23" s="18" t="n"/>
@@ -17018,7 +17024,7 @@
       <c r="EC42" s="18" t="n"/>
       <c r="ED42" s="18" t="n"/>
       <c r="EE42" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="EF42" s="18" t="n"/>
       <c r="EG42" s="18" t="n"/>
@@ -26350,7 +26356,9 @@
       </c>
       <c r="EC75" s="18" t="n"/>
       <c r="ED75" s="18" t="n"/>
-      <c r="EE75" s="18" t="n"/>
+      <c r="EE75" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EF75" s="18" t="n"/>
       <c r="EG75" s="18" t="n"/>
       <c r="EH75" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-06 21:11 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8357,7 +8357,9 @@
       <c r="EB12" s="18" t="n"/>
       <c r="EC12" s="18" t="n"/>
       <c r="ED12" s="18" t="n"/>
-      <c r="EE12" s="18" t="n"/>
+      <c r="EE12" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EF12" s="18" t="n"/>
       <c r="EG12" s="18" t="n"/>
       <c r="EH12" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-08 14:37 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8050,7 +8050,9 @@
       <c r="EE11" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="EF11" s="18" t="n"/>
+      <c r="EF11" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="EG11" s="18" t="n"/>
       <c r="EH11" s="18" t="n"/>
       <c r="EI11" s="18" t="n"/>
@@ -10983,7 +10985,9 @@
       <c r="EE21" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="EF21" s="18" t="n"/>
+      <c r="EF21" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="EG21" s="18" t="n"/>
       <c r="EH21" s="18" t="n"/>
       <c r="EI21" s="18" t="n"/>
@@ -13925,7 +13929,9 @@
       <c r="EE31" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="EF31" s="18" t="n"/>
+      <c r="EF31" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EG31" s="18" t="n"/>
       <c r="EH31" s="18" t="n"/>
       <c r="EI31" s="18" t="n"/>
@@ -16481,7 +16487,9 @@
       <c r="EC40" s="18" t="n"/>
       <c r="ED40" s="18" t="n"/>
       <c r="EE40" s="18" t="n"/>
-      <c r="EF40" s="18" t="n"/>
+      <c r="EF40" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EG40" s="18" t="n"/>
       <c r="EH40" s="18" t="n"/>
       <c r="EI40" s="18" t="n"/>
@@ -23815,7 +23823,9 @@
       <c r="EC66" s="18" t="n"/>
       <c r="ED66" s="18" t="n"/>
       <c r="EE66" s="18" t="n"/>
-      <c r="EF66" s="18" t="n"/>
+      <c r="EF66" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EG66" s="18" t="n"/>
       <c r="EH66" s="18" t="n"/>
       <c r="EI66" s="18" t="n"/>
@@ -26977,7 +26987,9 @@
       <c r="EC77" s="18" t="n"/>
       <c r="ED77" s="18" t="n"/>
       <c r="EE77" s="18" t="n"/>
-      <c r="EF77" s="18" t="n"/>
+      <c r="EF77" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="EG77" s="18" t="n"/>
       <c r="EH77" s="18" t="n"/>
       <c r="EI77" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-08 21:56 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8053,7 +8053,9 @@
       <c r="EF11" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="EG11" s="18" t="n"/>
+      <c r="EG11" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EH11" s="18" t="n"/>
       <c r="EI11" s="18" t="n"/>
       <c r="EJ11" s="18" t="n"/>
@@ -8363,7 +8365,9 @@
         <v>1</v>
       </c>
       <c r="EF12" s="18" t="n"/>
-      <c r="EG12" s="18" t="n"/>
+      <c r="EG12" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EH12" s="18" t="n"/>
       <c r="EI12" s="18" t="n"/>
       <c r="EJ12" s="18" t="n"/>
@@ -11593,7 +11597,9 @@
         <v>0.5</v>
       </c>
       <c r="EF23" s="18" t="n"/>
-      <c r="EG23" s="18" t="n"/>
+      <c r="EG23" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EH23" s="18" t="n"/>
       <c r="EI23" s="18" t="n"/>
       <c r="EJ23" s="18" t="n"/>
@@ -13932,7 +13938,9 @@
       <c r="EF31" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="EG31" s="18" t="n"/>
+      <c r="EG31" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EH31" s="18" t="n"/>
       <c r="EI31" s="18" t="n"/>
       <c r="EJ31" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-08 23:49 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8366,7 +8366,7 @@
       </c>
       <c r="EF12" s="18" t="n"/>
       <c r="EG12" s="18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="EH12" s="18" t="n"/>
       <c r="EI12" s="18" t="n"/>
@@ -11598,7 +11598,7 @@
       </c>
       <c r="EF23" s="18" t="n"/>
       <c r="EG23" s="18" t="n">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="EH23" s="18" t="n"/>
       <c r="EI23" s="18" t="n"/>
@@ -23834,7 +23834,9 @@
       <c r="EF66" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="EG66" s="18" t="n"/>
+      <c r="EG66" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="EH66" s="18" t="n"/>
       <c r="EI66" s="18" t="n"/>
       <c r="EJ66" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-09 21:08 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8368,7 +8368,9 @@
       <c r="EG12" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="EH12" s="18" t="n"/>
+      <c r="EH12" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="EI12" s="18" t="n"/>
       <c r="EJ12" s="18" t="n"/>
       <c r="EK12" s="18" t="n"/>
@@ -9236,7 +9238,9 @@
       <c r="EE15" s="18" t="n"/>
       <c r="EF15" s="18" t="n"/>
       <c r="EG15" s="18" t="n"/>
-      <c r="EH15" s="18" t="n"/>
+      <c r="EH15" s="18" t="n">
+        <v>3</v>
+      </c>
       <c r="EI15" s="18" t="n"/>
       <c r="EJ15" s="18" t="n"/>
       <c r="EK15" s="18" t="n"/>
@@ -13941,7 +13945,9 @@
       <c r="EG31" s="18" t="n">
         <v>0.5</v>
       </c>
-      <c r="EH31" s="18" t="n"/>
+      <c r="EH31" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EI31" s="18" t="n"/>
       <c r="EJ31" s="18" t="n"/>
       <c r="EK31" s="18" t="n"/>
@@ -16499,7 +16505,9 @@
         <v>1</v>
       </c>
       <c r="EG40" s="18" t="n"/>
-      <c r="EH40" s="18" t="n"/>
+      <c r="EH40" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EI40" s="18" t="n"/>
       <c r="EJ40" s="18" t="n"/>
       <c r="EK40" s="18" t="n"/>
@@ -23837,7 +23845,9 @@
       <c r="EG66" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="EH66" s="18" t="n"/>
+      <c r="EH66" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EI66" s="18" t="n"/>
       <c r="EJ66" s="18" t="n"/>
       <c r="EK66" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-14 22:18 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8373,7 +8373,9 @@
       </c>
       <c r="EI12" s="18" t="n"/>
       <c r="EJ12" s="18" t="n"/>
-      <c r="EK12" s="18" t="n"/>
+      <c r="EK12" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="EL12" s="18" t="n"/>
       <c r="EM12" s="18" t="n"/>
       <c r="EN12" s="18" t="n"/>
@@ -11607,7 +11609,9 @@
       <c r="EH23" s="18" t="n"/>
       <c r="EI23" s="18" t="n"/>
       <c r="EJ23" s="18" t="n"/>
-      <c r="EK23" s="18" t="n"/>
+      <c r="EK23" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EL23" s="18" t="n"/>
       <c r="EM23" s="18" t="n"/>
       <c r="EN23" s="18" t="n"/>
@@ -13950,7 +13954,9 @@
       </c>
       <c r="EI31" s="18" t="n"/>
       <c r="EJ31" s="18" t="n"/>
-      <c r="EK31" s="18" t="n"/>
+      <c r="EK31" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EL31" s="18" t="n"/>
       <c r="EM31" s="18" t="n"/>
       <c r="EN31" s="18" t="n"/>
@@ -23850,7 +23856,9 @@
       </c>
       <c r="EI66" s="18" t="n"/>
       <c r="EJ66" s="18" t="n"/>
-      <c r="EK66" s="18" t="n"/>
+      <c r="EK66" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EL66" s="18" t="n"/>
       <c r="EM66" s="18" t="n"/>
       <c r="EN66" s="18" t="n"/>
@@ -26398,7 +26406,9 @@
       <c r="EH75" s="18" t="n"/>
       <c r="EI75" s="18" t="n"/>
       <c r="EJ75" s="18" t="n"/>
-      <c r="EK75" s="18" t="n"/>
+      <c r="EK75" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EL75" s="18" t="n"/>
       <c r="EM75" s="18" t="n"/>
       <c r="EN75" s="18" t="n"/>
@@ -26733,7 +26743,9 @@
       <c r="EH76" s="18" t="n"/>
       <c r="EI76" s="18" t="n"/>
       <c r="EJ76" s="18" t="n"/>
-      <c r="EK76" s="18" t="n"/>
+      <c r="EK76" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EL76" s="18" t="n"/>
       <c r="EM76" s="18" t="n"/>
       <c r="EN76" s="18" t="n"/>
@@ -27014,7 +27026,9 @@
       <c r="EH77" s="18" t="n"/>
       <c r="EI77" s="18" t="n"/>
       <c r="EJ77" s="18" t="n"/>
-      <c r="EK77" s="18" t="n"/>
+      <c r="EK77" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EL77" s="18" t="n"/>
       <c r="EM77" s="18" t="n"/>
       <c r="EN77" s="18" t="n"/>

</xml_diff>

<commit_message>
Update: DSafarik_2026TimeTracking.xlsx [2026-07-14 22:20 UTC]
</commit_message>
<xml_diff>
--- a/DSafarik_2026TimeTracking.xlsx
+++ b/DSafarik_2026TimeTracking.xlsx
@@ -8372,7 +8372,9 @@
         <v>2</v>
       </c>
       <c r="EI12" s="18" t="n"/>
-      <c r="EJ12" s="18" t="n"/>
+      <c r="EJ12" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="EK12" s="18" t="n">
         <v>2</v>
       </c>
@@ -9806,7 +9808,9 @@
       <c r="EG17" s="18" t="n"/>
       <c r="EH17" s="18" t="n"/>
       <c r="EI17" s="18" t="n"/>
-      <c r="EJ17" s="18" t="n"/>
+      <c r="EJ17" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EK17" s="18" t="n"/>
       <c r="EL17" s="18" t="n"/>
       <c r="EM17" s="18" t="n"/>
@@ -13953,7 +13957,9 @@
         <v>1</v>
       </c>
       <c r="EI31" s="18" t="n"/>
-      <c r="EJ31" s="18" t="n"/>
+      <c r="EJ31" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="EK31" s="18" t="n">
         <v>1</v>
       </c>
@@ -14231,7 +14237,9 @@
       <c r="EG32" s="18" t="n"/>
       <c r="EH32" s="18" t="n"/>
       <c r="EI32" s="18" t="n"/>
-      <c r="EJ32" s="18" t="n"/>
+      <c r="EJ32" s="18" t="n">
+        <v>2</v>
+      </c>
       <c r="EK32" s="18" t="n"/>
       <c r="EL32" s="18" t="n"/>
       <c r="EM32" s="18" t="n"/>
@@ -14595,7 +14603,9 @@
       <c r="EG33" s="18" t="n"/>
       <c r="EH33" s="18" t="n"/>
       <c r="EI33" s="18" t="n"/>
-      <c r="EJ33" s="18" t="n"/>
+      <c r="EJ33" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EK33" s="18" t="n"/>
       <c r="EL33" s="18" t="n"/>
       <c r="EM33" s="18" t="n"/>
@@ -17064,7 +17074,9 @@
       <c r="EG42" s="18" t="n"/>
       <c r="EH42" s="18" t="n"/>
       <c r="EI42" s="18" t="n"/>
-      <c r="EJ42" s="18" t="n"/>
+      <c r="EJ42" s="18" t="n">
+        <v>1</v>
+      </c>
       <c r="EK42" s="18" t="n"/>
       <c r="EL42" s="18" t="n"/>
       <c r="EM42" s="18" t="n"/>
@@ -24432,7 +24444,9 @@
       <c r="EG68" s="18" t="n"/>
       <c r="EH68" s="18" t="n"/>
       <c r="EI68" s="18" t="n"/>
-      <c r="EJ68" s="18" t="n"/>
+      <c r="EJ68" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EK68" s="18" t="n"/>
       <c r="EL68" s="18" t="n"/>
       <c r="EM68" s="18" t="n"/>
@@ -25248,7 +25262,9 @@
       <c r="EG71" s="18" t="n"/>
       <c r="EH71" s="18" t="n"/>
       <c r="EI71" s="18" t="n"/>
-      <c r="EJ71" s="18" t="n"/>
+      <c r="EJ71" s="18" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EK71" s="18" t="n"/>
       <c r="EL71" s="18" t="n"/>
       <c r="EM71" s="18" t="n"/>

</xml_diff>